<commit_message>
Add game data and log files for users 22-33; Inserted the new field 'should_be_a_match';
</commit_message>
<xml_diff>
--- a/app/analysis/Questionnaire_results.xlsx
+++ b/app/analysis/Questionnaire_results.xlsx
@@ -8,6 +8,9 @@
   </bookViews>
   <sheets>
     <sheet name="PSI_scales" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="PSI_Results" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="PSI_PostHoc" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Trust_Results" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -431,7 +434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P21"/>
+  <dimension ref="A1:P33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -744,163 +747,163 @@
     </row>
     <row r="6">
       <c r="A6" s="3" t="n">
-        <v>2</v>
+        <v>21</v>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>CS0</t>
+          <t>CC</t>
         </is>
       </c>
       <c r="C6" s="3" t="n">
-        <v>1</v>
+        <v>1.75</v>
       </c>
       <c r="D6" s="3" t="n">
         <v>2</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>2.25</v>
+        <v>4</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>4</v>
+        <v>2.5</v>
       </c>
       <c r="G6" s="3" t="n">
         <v>2</v>
       </c>
       <c r="H6" s="3" t="n">
-        <v>2.5</v>
+        <v>2</v>
       </c>
       <c r="I6" s="3" t="n">
-        <v>1.8</v>
+        <v>2.6</v>
       </c>
       <c r="J6" s="3" t="n">
-        <v>3.8</v>
+        <v>2.8</v>
       </c>
       <c r="K6" s="3" t="n">
-        <v>2.2</v>
+        <v>2.8</v>
       </c>
       <c r="L6" s="3" t="n">
-        <v>2</v>
+        <v>2.8</v>
       </c>
       <c r="M6" s="3" t="n">
-        <v>2.8</v>
+        <v>2.6</v>
       </c>
       <c r="N6" s="3" t="n">
-        <v>3</v>
+        <v>1.4</v>
       </c>
       <c r="O6" s="3" t="n">
-        <v>1.8</v>
+        <v>3.6</v>
       </c>
       <c r="P6" s="3" t="n">
-        <v>1.4</v>
+        <v>3.4</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="n">
-        <v>7</v>
+        <v>26</v>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>CS0</t>
+          <t>CC</t>
         </is>
       </c>
       <c r="C7" s="3" t="n">
-        <v>3.25</v>
+        <v>4.25</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>3.25</v>
+        <v>4.5</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>3.5</v>
+        <v>4.75</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>1.75</v>
+        <v>4.5</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H7" s="3" t="n">
-        <v>1</v>
+        <v>4.75</v>
       </c>
       <c r="I7" s="3" t="n">
-        <v>3.4</v>
+        <v>5</v>
       </c>
       <c r="J7" s="3" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K7" s="3" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L7" s="3" t="n">
-        <v>3</v>
+        <v>4.6</v>
       </c>
       <c r="M7" s="3" t="n">
-        <v>3</v>
+        <v>4.4</v>
       </c>
       <c r="N7" s="3" t="n">
-        <v>3.4</v>
+        <v>5</v>
       </c>
       <c r="O7" s="3" t="n">
-        <v>2.8</v>
+        <v>4.8</v>
       </c>
       <c r="P7" s="3" t="n">
-        <v>1.6</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="n">
-        <v>12</v>
+        <v>31</v>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>CS0</t>
+          <t>CC</t>
         </is>
       </c>
       <c r="C8" s="3" t="n">
-        <v>2.5</v>
+        <v>1</v>
       </c>
       <c r="D8" s="3" t="n">
         <v>2</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>4</v>
+        <v>2.25</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>4.25</v>
+        <v>3</v>
       </c>
       <c r="H8" s="3" t="n">
-        <v>4.5</v>
+        <v>3</v>
       </c>
       <c r="I8" s="3" t="n">
-        <v>4.6</v>
+        <v>1</v>
       </c>
       <c r="J8" s="3" t="n">
-        <v>4.8</v>
+        <v>1</v>
       </c>
       <c r="K8" s="3" t="n">
-        <v>4.4</v>
+        <v>1</v>
       </c>
       <c r="L8" s="3" t="n">
-        <v>4.8</v>
+        <v>1</v>
       </c>
       <c r="M8" s="3" t="n">
-        <v>3.2</v>
+        <v>1</v>
       </c>
       <c r="N8" s="3" t="n">
-        <v>3.2</v>
+        <v>1</v>
       </c>
       <c r="O8" s="3" t="n">
-        <v>4.2</v>
+        <v>1</v>
       </c>
       <c r="P8" s="3" t="n">
-        <v>4.2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="n">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
@@ -908,671 +911,3387 @@
         </is>
       </c>
       <c r="C9" s="3" t="n">
-        <v>2</v>
+        <v>3.25</v>
       </c>
       <c r="D9" s="3" t="n">
-        <v>2</v>
+        <v>3.25</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>2.25</v>
+        <v>3.5</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>3</v>
+        <v>1.75</v>
       </c>
       <c r="G9" s="3" t="n">
-        <v>3.5</v>
+        <v>4</v>
       </c>
       <c r="H9" s="3" t="n">
-        <v>3.75</v>
+        <v>1</v>
       </c>
       <c r="I9" s="3" t="n">
-        <v>3</v>
+        <v>3.4</v>
       </c>
       <c r="J9" s="3" t="n">
         <v>3</v>
       </c>
       <c r="K9" s="3" t="n">
-        <v>3.8</v>
+        <v>3</v>
       </c>
       <c r="L9" s="3" t="n">
-        <v>3.6</v>
+        <v>3</v>
       </c>
       <c r="M9" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="N9" s="3" t="n">
         <v>3.4</v>
       </c>
-      <c r="N9" s="3" t="n">
-        <v>4</v>
-      </c>
       <c r="O9" s="3" t="n">
-        <v>3</v>
+        <v>2.8</v>
       </c>
       <c r="P9" s="3" t="n">
-        <v>3.4</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>CS1</t>
+          <t>CS0</t>
         </is>
       </c>
       <c r="C10" s="3" t="n">
-        <v>3.5</v>
+        <v>2.5</v>
       </c>
       <c r="D10" s="3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E10" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="F10" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="G10" s="3" t="n">
+        <v>4.25</v>
+      </c>
+      <c r="H10" s="3" t="n">
         <v>4.5</v>
       </c>
-      <c r="F10" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="G10" s="3" t="n">
-        <v>3.25</v>
-      </c>
-      <c r="H10" s="3" t="n">
-        <v>3</v>
-      </c>
       <c r="I10" s="3" t="n">
-        <v>4</v>
+        <v>4.6</v>
       </c>
       <c r="J10" s="3" t="n">
-        <v>2.4</v>
+        <v>4.8</v>
       </c>
       <c r="K10" s="3" t="n">
-        <v>3.6</v>
+        <v>4.4</v>
       </c>
       <c r="L10" s="3" t="n">
-        <v>3.6</v>
+        <v>4.8</v>
       </c>
       <c r="M10" s="3" t="n">
-        <v>1.6</v>
+        <v>3.2</v>
       </c>
       <c r="N10" s="3" t="n">
-        <v>2</v>
+        <v>3.2</v>
       </c>
       <c r="O10" s="3" t="n">
-        <v>4</v>
+        <v>4.2</v>
       </c>
       <c r="P10" s="3" t="n">
-        <v>3.8</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="n">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>CS1</t>
+          <t>CS0</t>
         </is>
       </c>
       <c r="C11" s="3" t="n">
-        <v>3.25</v>
+        <v>2</v>
       </c>
       <c r="D11" s="3" t="n">
-        <v>2.5</v>
+        <v>2</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>2.75</v>
+        <v>2.25</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>2.75</v>
+        <v>3</v>
       </c>
       <c r="G11" s="3" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="H11" s="3" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="I11" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="H11" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="I11" s="3" t="n">
-        <v>1.6</v>
-      </c>
       <c r="J11" s="3" t="n">
-        <v>1.6</v>
+        <v>3</v>
       </c>
       <c r="K11" s="3" t="n">
-        <v>1.8</v>
+        <v>3.8</v>
       </c>
       <c r="L11" s="3" t="n">
-        <v>2</v>
+        <v>3.6</v>
       </c>
       <c r="M11" s="3" t="n">
-        <v>2.6</v>
+        <v>3.4</v>
       </c>
       <c r="N11" s="3" t="n">
-        <v>2.4</v>
+        <v>4</v>
       </c>
       <c r="O11" s="3" t="n">
-        <v>2.8</v>
+        <v>3</v>
       </c>
       <c r="P11" s="3" t="n">
-        <v>2.6</v>
+        <v>3.4</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>CS1</t>
+          <t>CS0</t>
         </is>
       </c>
       <c r="C12" s="3" t="n">
-        <v>2.75</v>
+        <v>2.5</v>
       </c>
       <c r="D12" s="3" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="E12" s="3" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="F12" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="E12" s="3" t="n">
+      <c r="G12" s="3" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="H12" s="3" t="n">
         <v>2.5</v>
       </c>
-      <c r="F12" s="3" t="n">
-        <v>3.5</v>
-      </c>
-      <c r="G12" s="3" t="n">
-        <v>2.75</v>
-      </c>
-      <c r="H12" s="3" t="n">
-        <v>2.75</v>
-      </c>
       <c r="I12" s="3" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="J12" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="K12" s="3" t="n">
         <v>3.2</v>
       </c>
-      <c r="J12" s="3" t="n">
-        <v>3.4</v>
-      </c>
-      <c r="K12" s="3" t="n">
-        <v>2.6</v>
-      </c>
       <c r="L12" s="3" t="n">
-        <v>3.4</v>
+        <v>3.6</v>
       </c>
       <c r="M12" s="3" t="n">
-        <v>2.4</v>
+        <v>3.8</v>
       </c>
       <c r="N12" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="O12" s="3" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="P12" s="3" t="n">
         <v>3.2</v>
-      </c>
-      <c r="O12" s="3" t="n">
-        <v>3.4</v>
-      </c>
-      <c r="P12" s="3" t="n">
-        <v>3.4</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="n">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>CS1</t>
+          <t>CS0</t>
         </is>
       </c>
       <c r="C13" s="3" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D13" s="3" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E13" s="3" t="n">
         <v>4</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>2.75</v>
+        <v>4</v>
       </c>
       <c r="H13" s="3" t="n">
-        <v>2.5</v>
+        <v>4</v>
       </c>
       <c r="I13" s="3" t="n">
-        <v>2.4</v>
+        <v>3.4</v>
       </c>
       <c r="J13" s="3" t="n">
-        <v>2</v>
+        <v>4.4</v>
       </c>
       <c r="K13" s="3" t="n">
-        <v>2.6</v>
+        <v>4</v>
       </c>
       <c r="L13" s="3" t="n">
-        <v>2.2</v>
+        <v>4.4</v>
       </c>
       <c r="M13" s="3" t="n">
-        <v>2.6</v>
+        <v>4.4</v>
       </c>
       <c r="N13" s="3" t="n">
-        <v>2.6</v>
+        <v>3.2</v>
       </c>
       <c r="O13" s="3" t="n">
-        <v>3</v>
+        <v>3.4</v>
       </c>
       <c r="P13" s="3" t="n">
-        <v>2.8</v>
+        <v>3.4</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="n">
+        <v>32</v>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>CS0</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="B14" s="3" t="inlineStr">
-        <is>
-          <t>CI</t>
-        </is>
-      </c>
-      <c r="C14" s="3" t="n">
-        <v>2.75</v>
-      </c>
       <c r="D14" s="3" t="n">
-        <v>2</v>
+        <v>4.25</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>3.75</v>
+        <v>5</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>3.5</v>
+        <v>2.5</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H14" s="3" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="I14" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="I14" s="3" t="n">
+      <c r="J14" s="3" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="K14" s="3" t="n">
         <v>4.4</v>
       </c>
-      <c r="J14" s="3" t="n">
-        <v>3.2</v>
-      </c>
-      <c r="K14" s="3" t="n">
-        <v>4.2</v>
-      </c>
       <c r="L14" s="3" t="n">
-        <v>2.8</v>
+        <v>1.6</v>
       </c>
       <c r="M14" s="3" t="n">
-        <v>3</v>
+        <v>4.8</v>
       </c>
       <c r="N14" s="3" t="n">
-        <v>2.2</v>
+        <v>2.6</v>
       </c>
       <c r="O14" s="3" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="P14" s="3" t="n">
-        <v>3.6</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>CI</t>
+          <t>CS1</t>
         </is>
       </c>
       <c r="C15" s="3" t="n">
-        <v>2.5</v>
+        <v>3.5</v>
       </c>
       <c r="D15" s="3" t="n">
-        <v>2.5</v>
+        <v>3</v>
       </c>
       <c r="E15" s="3" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="F15" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="G15" s="3" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="H15" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="I15" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="F15" s="3" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="G15" s="3" t="n">
-        <v>3.5</v>
-      </c>
-      <c r="H15" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="I15" s="3" t="n">
-        <v>2.2</v>
-      </c>
       <c r="J15" s="3" t="n">
-        <v>2.8</v>
+        <v>2.4</v>
       </c>
       <c r="K15" s="3" t="n">
-        <v>2.8</v>
+        <v>3.6</v>
       </c>
       <c r="L15" s="3" t="n">
-        <v>2.4</v>
+        <v>3.6</v>
       </c>
       <c r="M15" s="3" t="n">
-        <v>3.2</v>
+        <v>1.6</v>
       </c>
       <c r="N15" s="3" t="n">
-        <v>1.8</v>
+        <v>2</v>
       </c>
       <c r="O15" s="3" t="n">
-        <v>3.4</v>
+        <v>4</v>
       </c>
       <c r="P15" s="3" t="n">
-        <v>2.4</v>
+        <v>3.8</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="n">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>CI</t>
+          <t>CS1</t>
         </is>
       </c>
       <c r="C16" s="3" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="D16" s="3" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="E16" s="3" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="F16" s="3" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="G16" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="D16" s="3" t="n">
-        <v>3.25</v>
-      </c>
-      <c r="E16" s="3" t="n">
-        <v>3.5</v>
-      </c>
-      <c r="F16" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="G16" s="3" t="n">
-        <v>3.25</v>
-      </c>
       <c r="H16" s="3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I16" s="3" t="n">
-        <v>3.4</v>
+        <v>1.6</v>
       </c>
       <c r="J16" s="3" t="n">
-        <v>2.2</v>
+        <v>1.6</v>
       </c>
       <c r="K16" s="3" t="n">
-        <v>3.6</v>
+        <v>1.8</v>
       </c>
       <c r="L16" s="3" t="n">
         <v>2</v>
       </c>
       <c r="M16" s="3" t="n">
-        <v>3.8</v>
+        <v>2.6</v>
       </c>
       <c r="N16" s="3" t="n">
-        <v>2.8</v>
+        <v>2.4</v>
       </c>
       <c r="O16" s="3" t="n">
         <v>2.8</v>
       </c>
       <c r="P16" s="3" t="n">
-        <v>1.8</v>
+        <v>2.6</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="n">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>CI</t>
+          <t>CS1</t>
         </is>
       </c>
       <c r="C17" s="3" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="D17" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E17" s="3" t="n">
         <v>2.5</v>
       </c>
-      <c r="D17" s="3" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="E17" s="3" t="n">
-        <v>3.75</v>
-      </c>
       <c r="F17" s="3" t="n">
-        <v>1</v>
+        <v>3.5</v>
       </c>
       <c r="G17" s="3" t="n">
-        <v>3.5</v>
+        <v>2.75</v>
       </c>
       <c r="H17" s="3" t="n">
-        <v>1</v>
+        <v>2.75</v>
       </c>
       <c r="I17" s="3" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="J17" s="3" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="K17" s="3" t="n">
         <v>2.6</v>
       </c>
-      <c r="J17" s="3" t="n">
-        <v>1.8</v>
-      </c>
-      <c r="K17" s="3" t="n">
+      <c r="L17" s="3" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="M17" s="3" t="n">
         <v>2.4</v>
       </c>
-      <c r="L17" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="M17" s="3" t="n">
-        <v>2.8</v>
-      </c>
       <c r="N17" s="3" t="n">
-        <v>2.8</v>
+        <v>3.2</v>
       </c>
       <c r="O17" s="3" t="n">
-        <v>1.6</v>
+        <v>3.4</v>
       </c>
       <c r="P17" s="3" t="n">
-        <v>1.4</v>
+        <v>3.4</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="n">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>II</t>
+          <t>CS1</t>
         </is>
       </c>
       <c r="C18" s="3" t="n">
-        <v>2.75</v>
+        <v>1</v>
       </c>
       <c r="D18" s="3" t="n">
-        <v>2.75</v>
+        <v>1</v>
       </c>
       <c r="E18" s="3" t="n">
         <v>4</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>1.75</v>
+        <v>2.75</v>
       </c>
       <c r="H18" s="3" t="n">
-        <v>1.5</v>
+        <v>2.5</v>
       </c>
       <c r="I18" s="3" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="J18" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="K18" s="3" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="L18" s="3" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="M18" s="3" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="N18" s="3" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="O18" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="P18" s="3" t="n">
         <v>2.8</v>
-      </c>
-      <c r="J18" s="3" t="n">
-        <v>2.8</v>
-      </c>
-      <c r="K18" s="3" t="n">
-        <v>3.2</v>
-      </c>
-      <c r="L18" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="M18" s="3" t="n">
-        <v>3.8</v>
-      </c>
-      <c r="N18" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="O18" s="3" t="n">
-        <v>2.6</v>
-      </c>
-      <c r="P18" s="3" t="n">
-        <v>2.2</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="n">
-        <v>10</v>
+        <v>23</v>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>II</t>
+          <t>CS1</t>
         </is>
       </c>
       <c r="C19" s="3" t="n">
-        <v>2</v>
+        <v>3.5</v>
       </c>
       <c r="D19" s="3" t="n">
-        <v>1.25</v>
+        <v>3.75</v>
       </c>
       <c r="E19" s="3" t="n">
-        <v>1</v>
+        <v>4.75</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>1.25</v>
+        <v>4.75</v>
       </c>
       <c r="G19" s="3" t="n">
-        <v>1.25</v>
+        <v>4.5</v>
       </c>
       <c r="H19" s="3" t="n">
-        <v>1.5</v>
+        <v>4.5</v>
       </c>
       <c r="I19" s="3" t="n">
-        <v>2.2</v>
+        <v>3.2</v>
       </c>
       <c r="J19" s="3" t="n">
-        <v>1.8</v>
+        <v>3</v>
       </c>
       <c r="K19" s="3" t="n">
-        <v>1.6</v>
+        <v>3</v>
       </c>
       <c r="L19" s="3" t="n">
-        <v>1.4</v>
+        <v>2.8</v>
       </c>
       <c r="M19" s="3" t="n">
-        <v>1.6</v>
+        <v>4</v>
       </c>
       <c r="N19" s="3" t="n">
-        <v>1.8</v>
+        <v>4</v>
       </c>
       <c r="O19" s="3" t="n">
-        <v>1.2</v>
+        <v>3</v>
       </c>
       <c r="P19" s="3" t="n">
-        <v>1.6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="n">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>II</t>
+          <t>CS1</t>
         </is>
       </c>
       <c r="C20" s="3" t="n">
-        <v>1.75</v>
+        <v>2.5</v>
       </c>
       <c r="D20" s="3" t="n">
         <v>1.75</v>
       </c>
       <c r="E20" s="3" t="n">
-        <v>1</v>
+        <v>4.75</v>
       </c>
       <c r="F20" s="3" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G20" s="3" t="n">
-        <v>1.75</v>
+        <v>4.5</v>
       </c>
       <c r="H20" s="3" t="n">
-        <v>1.5</v>
+        <v>4.5</v>
       </c>
       <c r="I20" s="3" t="n">
-        <v>1.4</v>
+        <v>3</v>
       </c>
       <c r="J20" s="3" t="n">
-        <v>1.2</v>
+        <v>3.6</v>
       </c>
       <c r="K20" s="3" t="n">
-        <v>2</v>
+        <v>3.8</v>
       </c>
       <c r="L20" s="3" t="n">
-        <v>1.6</v>
+        <v>4.2</v>
       </c>
       <c r="M20" s="3" t="n">
         <v>2.2</v>
       </c>
       <c r="N20" s="3" t="n">
-        <v>2</v>
+        <v>1.8</v>
       </c>
       <c r="O20" s="3" t="n">
-        <v>1.2</v>
+        <v>3.8</v>
       </c>
       <c r="P20" s="3" t="n">
-        <v>1</v>
+        <v>3.6</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="n">
+        <v>33</v>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>CS1</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="D21" s="3" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="E21" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="F21" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="G21" s="3" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="H21" s="3" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="I21" s="3" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="J21" s="3" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="K21" s="3" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="L21" s="3" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="M21" s="3" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="N21" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="O21" s="3" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="P21" s="3" t="n">
+        <v>2.4</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>CI</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="D22" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E22" s="3" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="F22" s="3" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="G22" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="H22" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="I22" s="3" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="J22" s="3" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="K22" s="3" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="L22" s="3" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="M22" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="N22" s="3" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="O22" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="P22" s="3" t="n">
+        <v>3.6</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>CI</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="D23" s="3" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="E23" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="F23" s="3" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="G23" s="3" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="H23" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="I23" s="3" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="J23" s="3" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="K23" s="3" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="L23" s="3" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="M23" s="3" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="N23" s="3" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="O23" s="3" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="P23" s="3" t="n">
+        <v>2.4</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>CI</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="D24" s="3" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="E24" s="3" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="F24" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="G24" s="3" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="H24" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="I24" s="3" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="J24" s="3" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="K24" s="3" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="L24" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="M24" s="3" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="N24" s="3" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="O24" s="3" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="P24" s="3" t="n">
+        <v>1.8</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="n">
+        <v>19</v>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>CI</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="D25" s="3" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="E25" s="3" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="F25" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G25" s="3" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="H25" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="I25" s="3" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="J25" s="3" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="K25" s="3" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="L25" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="M25" s="3" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="N25" s="3" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="O25" s="3" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="P25" s="3" t="n">
+        <v>1.4</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="n">
+        <v>24</v>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>CI</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="D26" s="3" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="E26" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="F26" s="3" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="G26" s="3" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="H26" s="3" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="I26" s="3" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="J26" s="3" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="K26" s="3" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="L26" s="3" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="M26" s="3" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="N26" s="3" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="O26" s="3" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="P26" s="3" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="n">
+        <v>29</v>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>CI</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="D27" s="3" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="E27" s="3" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="F27" s="3" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="G27" s="3" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="H27" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="I27" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="J27" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="K27" s="3" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="L27" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="M27" s="3" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="N27" s="3" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="O27" s="3" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="P27" s="3" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>II</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="D28" s="3" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="E28" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="F28" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="G28" s="3" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="H28" s="3" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="I28" s="3" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="J28" s="3" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="K28" s="3" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="L28" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="M28" s="3" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="N28" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="O28" s="3" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="P28" s="3" t="n">
+        <v>2.2</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>II</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D29" s="3" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="E29" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F29" s="3" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="G29" s="3" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="H29" s="3" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="I29" s="3" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="J29" s="3" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="K29" s="3" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="L29" s="3" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="M29" s="3" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="N29" s="3" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="O29" s="3" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="P29" s="3" t="n">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>II</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="D30" s="3" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="E30" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F30" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G30" s="3" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="H30" s="3" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="I30" s="3" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="J30" s="3" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="K30" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="L30" s="3" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="M30" s="3" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="N30" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="O30" s="3" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="P30" s="3" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="n">
         <v>20</v>
       </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>II</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="D31" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E31" s="3" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="F31" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="G31" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="H31" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="I31" s="3" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="J31" s="3" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="K31" s="3" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="L31" s="3" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="M31" s="3" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="N31" s="3" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="O31" s="3" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="P31" s="3" t="n">
+        <v>2.8</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="n">
+        <v>25</v>
+      </c>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>II</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D32" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E32" s="3" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F32" s="3" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="G32" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="H32" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="I32" s="3" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="J32" s="3" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="K32" s="3" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="L32" s="3" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="M32" s="3" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="N32" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="O32" s="3" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="P32" s="3" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>II</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="D33" s="3" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="E33" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="F33" s="3" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="G33" s="3" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="H33" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="I33" s="3" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="J33" s="3" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="K33" s="3" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="L33" s="3" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="M33" s="3" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="N33" s="3" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="O33" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="P33" s="3" t="n">
+        <v>2.2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F28"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="17" customWidth="1" min="1" max="1"/>
+    <col width="23" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="25" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Analisi</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Variabile/Condizione</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Test Utilizzato</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Statistica</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>p-value</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>Significativo (p&lt;0.05)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>Tra Condizioni</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>SOC_D</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>ANOVA</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>0.3516893171488348</v>
+      </c>
+      <c r="E2" s="3" t="n">
+        <v>0.8405365027216767</v>
+      </c>
+      <c r="F2" s="3" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Tra Condizioni</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>SOC_M</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>ANOVA</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>1.314948117097306</v>
+      </c>
+      <c r="E3" s="3" t="n">
+        <v>0.2895873486983646</v>
+      </c>
+      <c r="F3" s="3" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Tra Condizioni</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>HLP_D</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Kruskal-Wallis</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>6.84552223996246</v>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>0.1442803595169977</v>
+      </c>
+      <c r="F4" s="3" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Tra Condizioni</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>HLP_M</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Kruskal-Wallis</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>8.368156484172905</v>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>0.07898587893462915</v>
+      </c>
+      <c r="F5" s="3" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Tra Condizioni</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>TRU_D</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Kruskal-Wallis</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="n">
+        <v>12.79907762919812</v>
+      </c>
+      <c r="E6" s="3" t="n">
+        <v>0.01230042900591252</v>
+      </c>
+      <c r="F6" s="3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Tra Condizioni</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>TRU_M</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>ANOVA</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>2.788053031972434</v>
+      </c>
+      <c r="E7" s="3" t="n">
+        <v>0.04646896518267722</v>
+      </c>
+      <c r="F7" s="3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr"/>
+      <c r="B8" s="3" t="inlineStr"/>
+      <c r="C8" s="3" t="inlineStr"/>
+      <c r="D8" s="3" t="inlineStr"/>
+      <c r="E8" s="3" t="inlineStr"/>
+      <c r="F8" s="3" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>Geo vs Math</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>SOC in CC</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>T-test Accoppiato</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="n">
+        <v>-2.517439175034821</v>
+      </c>
+      <c r="E9" s="3" t="n">
+        <v>0.04544403991949149</v>
+      </c>
+      <c r="F9" s="3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>Geo vs Math</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>HLP in CC</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Wilcoxon</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" s="3" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="F10" s="3" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>Geo vs Math</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>TRU in CC</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>T-test Accoppiato</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="n">
+        <v>-1.111437860452423</v>
+      </c>
+      <c r="E11" s="3" t="n">
+        <v>0.3089213661430785</v>
+      </c>
+      <c r="F11" s="3" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr"/>
+      <c r="B12" s="3" t="inlineStr"/>
+      <c r="C12" s="3" t="inlineStr"/>
+      <c r="D12" s="3" t="inlineStr"/>
+      <c r="E12" s="3" t="inlineStr"/>
+      <c r="F12" s="3" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Geo vs Math</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>SOC in CS0</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>Wilcoxon</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E13" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F13" s="3" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>Geo vs Math</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>HLP in CS0</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>T-test Accoppiato</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="n">
+        <v>1.242259987499883</v>
+      </c>
+      <c r="E14" s="3" t="n">
+        <v>0.2692267472099367</v>
+      </c>
+      <c r="F14" s="3" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Geo vs Math</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>TRU in CS0</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>T-test Accoppiato</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="n">
+        <v>1.706574098530288</v>
+      </c>
+      <c r="E15" s="3" t="n">
+        <v>0.1486119507797838</v>
+      </c>
+      <c r="F15" s="3" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr"/>
+      <c r="B16" s="3" t="inlineStr"/>
+      <c r="C16" s="3" t="inlineStr"/>
+      <c r="D16" s="3" t="inlineStr"/>
+      <c r="E16" s="3" t="inlineStr"/>
+      <c r="F16" s="3" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>Geo vs Math</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>SOC in CS1</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>T-test Accoppiato</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="n">
+        <v>1.527525231651947</v>
+      </c>
+      <c r="E17" s="3" t="n">
+        <v>0.1774888324162401</v>
+      </c>
+      <c r="F17" s="3" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>Geo vs Math</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>HLP in CS1</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>T-test Accoppiato</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="n">
+        <v>1.030114251517296</v>
+      </c>
+      <c r="E18" s="3" t="n">
+        <v>0.3426799101911869</v>
+      </c>
+      <c r="F18" s="3" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>Geo vs Math</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>TRU in CS1</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>Wilcoxon</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E19" s="3" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="F19" s="3" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr"/>
+      <c r="B20" s="3" t="inlineStr"/>
+      <c r="C20" s="3" t="inlineStr"/>
+      <c r="D20" s="3" t="inlineStr"/>
+      <c r="E20" s="3" t="inlineStr"/>
+      <c r="F20" s="3" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>Geo vs Math</t>
+        </is>
+      </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
+          <t>SOC in CI</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>T-test Accoppiato</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E21" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F21" s="3" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>Geo vs Math</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>HLP in CI</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>T-test Accoppiato</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="n">
+        <v>3.585685828003181</v>
+      </c>
+      <c r="E22" s="3" t="n">
+        <v>0.01577977641028941</v>
+      </c>
+      <c r="F22" s="3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>Geo vs Math</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>TRU in CI</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>T-test Accoppiato</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="n">
+        <v>1.846036752151603</v>
+      </c>
+      <c r="E23" s="3" t="n">
+        <v>0.1241798811672948</v>
+      </c>
+      <c r="F23" s="3" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr"/>
+      <c r="B24" s="3" t="inlineStr"/>
+      <c r="C24" s="3" t="inlineStr"/>
+      <c r="D24" s="3" t="inlineStr"/>
+      <c r="E24" s="3" t="inlineStr"/>
+      <c r="F24" s="3" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>Geo vs Math</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>SOC in II</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>Wilcoxon</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E25" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F25" s="3" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>Geo vs Math</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>HLP in II</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>T-test Accoppiato</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="n">
+        <v>0.9999999999999999</v>
+      </c>
+      <c r="E26" s="3" t="n">
+        <v>0.3632174676491224</v>
+      </c>
+      <c r="F26" s="3" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>Geo vs Math</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>TRU in II</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>T-test Accoppiato</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="n">
+        <v>-0.1910401799752175</v>
+      </c>
+      <c r="E27" s="3" t="n">
+        <v>0.8560092340671523</v>
+      </c>
+      <c r="F27" s="3" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr"/>
+      <c r="B28" s="3" t="inlineStr"/>
+      <c r="C28" s="3" t="inlineStr"/>
+      <c r="D28" s="3" t="inlineStr"/>
+      <c r="E28" s="3" t="inlineStr"/>
+      <c r="F28" s="3" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="23" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>p-value_corretto</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Variabile</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>Significativo</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>Test Post-Hoc</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>CC</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>CI</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="n">
+        <v>0.8282200262105117</v>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>TRU_D</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>Holm</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>CC</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>CS0</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="n">
+        <v>0.08344982949310291</v>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>TRU_D</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>Holm</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>CC</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>CS1</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>0.9484912846303624</v>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>TRU_D</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Holm</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>CC</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
           <t>II</t>
         </is>
       </c>
+      <c r="C5" s="3" t="n">
+        <v>0.02154030616308052</v>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>TRU_D</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>Holm</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>CI</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>CS0</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="n">
+        <v>0.03975834963909074</v>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>TRU_D</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>Holm</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>CI</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>CS1</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="n">
+        <v>0.8279813594784788</v>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>TRU_D</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>Holm</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>CI</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>II</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="n">
+        <v>0.02862006611735959</v>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>TRU_D</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>Holm</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>CS0</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>CS1</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="n">
+        <v>0.4275564756355391</v>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>TRU_D</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>Holm</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>CS0</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>II</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="n">
+        <v>0.007471721114744322</v>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>TRU_D</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>Holm</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>CS1</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>II</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="n">
+        <v>0.0173060655501628</v>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>TRU_D</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>Holm</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>CC</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>CI</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="n">
+        <v>0.2856568201695698</v>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>TRU_M</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>Tukey</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>CC</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>CS0</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="n">
+        <v>0.8825406577561964</v>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>TRU_M</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>Tukey</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>CC</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>CS1</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="n">
+        <v>0.9968785967175552</v>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>TRU_M</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>Tukey</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>CC</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>II</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="n">
+        <v>0.05885005189004744</v>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>TRU_M</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>Tukey</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>CI</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>CS0</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="n">
+        <v>0.8316841271375279</v>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>TRU_M</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>Tukey</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>CI</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>CS1</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="n">
+        <v>0.4579416519523574</v>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>TRU_M</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>Tukey</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>CI</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>II</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="n">
+        <v>0.9283490927481413</v>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>TRU_M</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>Tukey</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>CS0</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>CS1</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="n">
+        <v>0.9735579043511582</v>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>TRU_M</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>Tukey</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>CS0</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>II</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="n">
+        <v>0.3694414478318331</v>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>TRU_M</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>Tukey</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>CS1</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>II</t>
+        </is>
+      </c>
       <c r="C21" s="3" t="n">
-        <v>3</v>
+        <v>0.1162825157171983</v>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>TRU_M</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>Tukey</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F35"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="17" customWidth="1" min="1" max="1"/>
+    <col width="23" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="23" customWidth="1" min="5" max="5"/>
+    <col width="25" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Analisi</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Variabile/Condizione</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Test Utilizzato</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Statistica</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>p-value</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>Significativo (p&lt;0.05)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>Tra Condizioni</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>PR_D</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>ANOVA</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>2.239069010656735</v>
+      </c>
+      <c r="E2" s="3" t="n">
+        <v>0.0912444399612828</v>
+      </c>
+      <c r="F2" s="3" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Tra Condizioni</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>PR_M</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>ANOVA</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>1.493848014011183</v>
+      </c>
+      <c r="E3" s="3" t="n">
+        <v>0.2318460388470296</v>
+      </c>
+      <c r="F3" s="3" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Tra Condizioni</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>PTC_D</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>ANOVA</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>1.260066099278524</v>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>0.3098713513253112</v>
+      </c>
+      <c r="F4" s="3" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Tra Condizioni</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>PTC_M</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>ANOVA</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>2.425918859355659</v>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>0.07238754512904651</v>
+      </c>
+      <c r="F5" s="3" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Tra Condizioni</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>PU_D</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>ANOVA</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="n">
+        <v>1.966387446908919</v>
+      </c>
+      <c r="E6" s="3" t="n">
+        <v>0.1282436441057686</v>
+      </c>
+      <c r="F6" s="3" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Tra Condizioni</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>PU_M</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>ANOVA</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>0.9072981804558573</v>
+      </c>
+      <c r="E7" s="3" t="n">
+        <v>0.4736804679037702</v>
+      </c>
+      <c r="F7" s="3" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>Tra Condizioni</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>F_D</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>ANOVA</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="n">
+        <v>2.354617214532873</v>
+      </c>
+      <c r="E8" s="3" t="n">
+        <v>0.07905770882292266</v>
+      </c>
+      <c r="F8" s="3" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>Tra Condizioni</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>F_M</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>ANOVA</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="n">
+        <v>2.492610010077259</v>
+      </c>
+      <c r="E9" s="3" t="n">
+        <v>0.0666750999068324</v>
+      </c>
+      <c r="F9" s="3" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr"/>
+      <c r="B10" s="3" t="inlineStr"/>
+      <c r="C10" s="3" t="inlineStr"/>
+      <c r="D10" s="3" t="inlineStr"/>
+      <c r="E10" s="3" t="inlineStr"/>
+      <c r="F10" s="3" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>Geo vs Math</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>PR in CC</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>T-test Accoppiato</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="n">
+        <v>-0.8323148993037752</v>
+      </c>
+      <c r="E11" s="3" t="n">
+        <v>0.4370983363053137</v>
+      </c>
+      <c r="F11" s="3" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>Geo vs Math</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>PTC in CC</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>T-test Accoppiato</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="n">
+        <v>-0.8293962196513643</v>
+      </c>
+      <c r="E12" s="3" t="n">
+        <v>0.438624415622445</v>
+      </c>
+      <c r="F12" s="3" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Geo vs Math</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>PU in CC</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>T-test Accoppiato</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="n">
+        <v>0.6333004963811245</v>
+      </c>
+      <c r="E13" s="3" t="n">
+        <v>0.549899173505021</v>
+      </c>
+      <c r="F13" s="3" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>Geo vs Math</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>F in CC</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>T-test Accoppiato</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="n">
+        <v>0.1786474002526238</v>
+      </c>
+      <c r="E14" s="3" t="n">
+        <v>0.8640941349883791</v>
+      </c>
+      <c r="F14" s="3" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr"/>
+      <c r="B15" s="3" t="inlineStr"/>
+      <c r="C15" s="3" t="inlineStr"/>
+      <c r="D15" s="3" t="inlineStr"/>
+      <c r="E15" s="3" t="inlineStr"/>
+      <c r="F15" s="3" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>Geo vs Math</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>PR in CS0</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>T-test Accoppiato</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="n">
+        <v>0.8103965430069947</v>
+      </c>
+      <c r="E16" s="3" t="n">
+        <v>0.4545388771419559</v>
+      </c>
+      <c r="F16" s="3" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>Geo vs Math</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>PTC in CS0</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>Wilcoxon</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="E17" s="3" t="n">
+        <v>0.8125</v>
+      </c>
+      <c r="F17" s="3" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>Geo vs Math</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>PU in CS0</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>T-test Accoppiato</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="n">
+        <v>0.817623560871883</v>
+      </c>
+      <c r="E18" s="3" t="n">
+        <v>0.4507615688534394</v>
+      </c>
+      <c r="F18" s="3" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>Geo vs Math</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>F in CS0</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>Wilcoxon</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="E19" s="3" t="n">
+        <v>0.375</v>
+      </c>
+      <c r="F19" s="3" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr"/>
+      <c r="B20" s="3" t="inlineStr"/>
+      <c r="C20" s="3" t="inlineStr"/>
+      <c r="D20" s="3" t="inlineStr"/>
+      <c r="E20" s="3" t="inlineStr"/>
+      <c r="F20" s="3" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>Geo vs Math</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>PR in CS1</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>T-test Accoppiato</t>
+        </is>
       </c>
       <c r="D21" s="3" t="n">
-        <v>3</v>
+        <v>0.8798826901281195</v>
       </c>
       <c r="E21" s="3" t="n">
-        <v>3.25</v>
-      </c>
-      <c r="F21" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="G21" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="H21" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="I21" s="3" t="n">
-        <v>1.8</v>
-      </c>
-      <c r="J21" s="3" t="n">
-        <v>2.6</v>
-      </c>
-      <c r="K21" s="3" t="n">
-        <v>2.8</v>
-      </c>
-      <c r="L21" s="3" t="n">
-        <v>3.2</v>
-      </c>
-      <c r="M21" s="3" t="n">
-        <v>2.8</v>
-      </c>
-      <c r="N21" s="3" t="n">
-        <v>2.4</v>
-      </c>
-      <c r="O21" s="3" t="n">
-        <v>2.6</v>
-      </c>
-      <c r="P21" s="3" t="n">
-        <v>2.8</v>
-      </c>
+        <v>0.412773025377815</v>
+      </c>
+      <c r="F21" s="3" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>Geo vs Math</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>PTC in CS1</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>T-test Accoppiato</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="n">
+        <v>-0.547722557505167</v>
+      </c>
+      <c r="E22" s="3" t="n">
+        <v>0.6036450565101357</v>
+      </c>
+      <c r="F22" s="3" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>Geo vs Math</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>PU in CS1</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>T-test Accoppiato</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="n">
+        <v>-0.7604691006293732</v>
+      </c>
+      <c r="E23" s="3" t="n">
+        <v>0.4757860843342303</v>
+      </c>
+      <c r="F23" s="3" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>Geo vs Math</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>F in CS1</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>T-test Accoppiato</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="n">
+        <v>3.286335345030996</v>
+      </c>
+      <c r="E24" s="3" t="n">
+        <v>0.01668998431583146</v>
+      </c>
+      <c r="F24" s="3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr"/>
+      <c r="B25" s="3" t="inlineStr"/>
+      <c r="C25" s="3" t="inlineStr"/>
+      <c r="D25" s="3" t="inlineStr"/>
+      <c r="E25" s="3" t="inlineStr"/>
+      <c r="F25" s="3" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>Geo vs Math</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>PR in CI</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>T-test Accoppiato</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="n">
+        <v>1.992633492465215</v>
+      </c>
+      <c r="E26" s="3" t="n">
+        <v>0.102903179695228</v>
+      </c>
+      <c r="F26" s="3" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>Geo vs Math</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>PTC in CI</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>T-test Accoppiato</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="n">
+        <v>5.196152422706632</v>
+      </c>
+      <c r="E27" s="3" t="n">
+        <v>0.003478165115286503</v>
+      </c>
+      <c r="F27" s="3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>Geo vs Math</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>PU in CI</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>T-test Accoppiato</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="n">
+        <v>2.938769068226293</v>
+      </c>
+      <c r="E28" s="3" t="n">
+        <v>0.03230268845013829</v>
+      </c>
+      <c r="F28" s="3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>Geo vs Math</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>F in CI</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>T-test Accoppiato</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="n">
+        <v>3.415650255319866</v>
+      </c>
+      <c r="E29" s="3" t="n">
+        <v>0.01892712407194564</v>
+      </c>
+      <c r="F29" s="3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr"/>
+      <c r="B30" s="3" t="inlineStr"/>
+      <c r="C30" s="3" t="inlineStr"/>
+      <c r="D30" s="3" t="inlineStr"/>
+      <c r="E30" s="3" t="inlineStr"/>
+      <c r="F30" s="3" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>Geo vs Math</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>PR in II</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>T-test Accoppiato</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="n">
+        <v>-1.035098339013531</v>
+      </c>
+      <c r="E31" s="3" t="n">
+        <v>0.3480661939250909</v>
+      </c>
+      <c r="F31" s="3" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="inlineStr">
+        <is>
+          <t>Geo vs Math</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>PTC in II</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>T-test Accoppiato</t>
+        </is>
+      </c>
+      <c r="D32" s="3" t="n">
+        <v>0.5906244232186181</v>
+      </c>
+      <c r="E32" s="3" t="n">
+        <v>0.5804564345825868</v>
+      </c>
+      <c r="F32" s="3" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t>Geo vs Math</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>PU in II</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>T-test Accoppiato</t>
+        </is>
+      </c>
+      <c r="D33" s="3" t="n">
+        <v>-0.2161688505835586</v>
+      </c>
+      <c r="E33" s="3" t="n">
+        <v>0.8373985197577309</v>
+      </c>
+      <c r="F33" s="3" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>Geo vs Math</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>F in II</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>T-test Accoppiato</t>
+        </is>
+      </c>
+      <c r="D34" s="3" t="n">
+        <v>0.7453559924999299</v>
+      </c>
+      <c r="E34" s="3" t="n">
+        <v>0.4895897445644272</v>
+      </c>
+      <c r="F34" s="3" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="inlineStr"/>
+      <c r="B35" s="3" t="inlineStr"/>
+      <c r="C35" s="3" t="inlineStr"/>
+      <c r="D35" s="3" t="inlineStr"/>
+      <c r="E35" s="3" t="inlineStr"/>
+      <c r="F35" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
new partecipants added; fixed field of csv
</commit_message>
<xml_diff>
--- a/app/analysis/Questionnaire_results.xlsx
+++ b/app/analysis/Questionnaire_results.xlsx
@@ -434,7 +434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P35"/>
+  <dimension ref="A1:P41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -903,111 +903,111 @@
     </row>
     <row r="9">
       <c r="A9" s="3" t="n">
-        <v>7</v>
+        <v>36</v>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>CS0</t>
+          <t>CC</t>
         </is>
       </c>
       <c r="C9" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="D9" s="3" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="E9" s="3" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="F9" s="3" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="G9" s="3" t="n">
         <v>3.25</v>
       </c>
-      <c r="D9" s="3" t="n">
-        <v>3.25</v>
-      </c>
-      <c r="E9" s="3" t="n">
+      <c r="H9" s="3" t="n">
         <v>3.5</v>
       </c>
-      <c r="F9" s="3" t="n">
-        <v>1.75</v>
-      </c>
-      <c r="G9" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="H9" s="3" t="n">
-        <v>1</v>
-      </c>
       <c r="I9" s="3" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="J9" s="3" t="n">
         <v>3.4</v>
       </c>
-      <c r="J9" s="3" t="n">
-        <v>3</v>
-      </c>
       <c r="K9" s="3" t="n">
-        <v>3</v>
+        <v>3.4</v>
       </c>
       <c r="L9" s="3" t="n">
-        <v>3</v>
+        <v>2.8</v>
       </c>
       <c r="M9" s="3" t="n">
-        <v>3</v>
+        <v>3.6</v>
       </c>
       <c r="N9" s="3" t="n">
-        <v>3.4</v>
+        <v>3.8</v>
       </c>
       <c r="O9" s="3" t="n">
         <v>2.8</v>
       </c>
       <c r="P9" s="3" t="n">
-        <v>1.6</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="n">
-        <v>12</v>
+        <v>41</v>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>CS0</t>
+          <t>CC</t>
         </is>
       </c>
       <c r="C10" s="3" t="n">
-        <v>2.5</v>
+        <v>3.25</v>
       </c>
       <c r="D10" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>4</v>
+        <v>3.75</v>
       </c>
       <c r="F10" s="3" t="n">
         <v>4</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>4.25</v>
+        <v>3</v>
       </c>
       <c r="H10" s="3" t="n">
-        <v>4.5</v>
+        <v>3</v>
       </c>
       <c r="I10" s="3" t="n">
-        <v>4.6</v>
+        <v>2.4</v>
       </c>
       <c r="J10" s="3" t="n">
-        <v>4.8</v>
+        <v>3.4</v>
       </c>
       <c r="K10" s="3" t="n">
-        <v>4.4</v>
+        <v>3.8</v>
       </c>
       <c r="L10" s="3" t="n">
-        <v>4.8</v>
+        <v>3.8</v>
       </c>
       <c r="M10" s="3" t="n">
-        <v>3.2</v>
+        <v>2.4</v>
       </c>
       <c r="N10" s="3" t="n">
-        <v>3.2</v>
+        <v>2.8</v>
       </c>
       <c r="O10" s="3" t="n">
-        <v>4.2</v>
+        <v>2.2</v>
       </c>
       <c r="P10" s="3" t="n">
-        <v>4.2</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="n">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
@@ -1015,51 +1015,51 @@
         </is>
       </c>
       <c r="C11" s="3" t="n">
-        <v>2</v>
+        <v>3.25</v>
       </c>
       <c r="D11" s="3" t="n">
-        <v>2</v>
+        <v>3.25</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>2.25</v>
+        <v>3.5</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>3</v>
+        <v>1.75</v>
       </c>
       <c r="G11" s="3" t="n">
-        <v>3.5</v>
+        <v>4</v>
       </c>
       <c r="H11" s="3" t="n">
-        <v>3.75</v>
+        <v>1</v>
       </c>
       <c r="I11" s="3" t="n">
-        <v>3</v>
+        <v>3.4</v>
       </c>
       <c r="J11" s="3" t="n">
         <v>3</v>
       </c>
       <c r="K11" s="3" t="n">
-        <v>3.8</v>
+        <v>3</v>
       </c>
       <c r="L11" s="3" t="n">
-        <v>3.6</v>
+        <v>3</v>
       </c>
       <c r="M11" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="N11" s="3" t="n">
         <v>3.4</v>
       </c>
-      <c r="N11" s="3" t="n">
-        <v>4</v>
-      </c>
       <c r="O11" s="3" t="n">
-        <v>3</v>
+        <v>2.8</v>
       </c>
       <c r="P11" s="3" t="n">
-        <v>3.4</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="n">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
@@ -1070,48 +1070,48 @@
         <v>2.5</v>
       </c>
       <c r="D12" s="3" t="n">
-        <v>2.5</v>
+        <v>2</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>3.25</v>
+        <v>4</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>3.5</v>
+        <v>4.25</v>
       </c>
       <c r="H12" s="3" t="n">
-        <v>2.5</v>
+        <v>4.5</v>
       </c>
       <c r="I12" s="3" t="n">
-        <v>3.4</v>
+        <v>4.6</v>
       </c>
       <c r="J12" s="3" t="n">
-        <v>3</v>
+        <v>4.8</v>
       </c>
       <c r="K12" s="3" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="L12" s="3" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="M12" s="3" t="n">
         <v>3.2</v>
       </c>
-      <c r="L12" s="3" t="n">
-        <v>3.6</v>
-      </c>
-      <c r="M12" s="3" t="n">
-        <v>3.8</v>
-      </c>
       <c r="N12" s="3" t="n">
-        <v>4</v>
+        <v>3.2</v>
       </c>
       <c r="O12" s="3" t="n">
-        <v>3.6</v>
+        <v>4.2</v>
       </c>
       <c r="P12" s="3" t="n">
-        <v>3.2</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="n">
-        <v>27</v>
+        <v>17</v>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
@@ -1119,43 +1119,43 @@
         </is>
       </c>
       <c r="C13" s="3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D13" s="3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E13" s="3" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="F13" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="G13" s="3" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="H13" s="3" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="I13" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="J13" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="K13" s="3" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="L13" s="3" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="M13" s="3" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="N13" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="F13" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="G13" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="H13" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="I13" s="3" t="n">
-        <v>3.4</v>
-      </c>
-      <c r="J13" s="3" t="n">
-        <v>4.4</v>
-      </c>
-      <c r="K13" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="L13" s="3" t="n">
-        <v>4.4</v>
-      </c>
-      <c r="M13" s="3" t="n">
-        <v>4.4</v>
-      </c>
-      <c r="N13" s="3" t="n">
-        <v>3.2</v>
-      </c>
       <c r="O13" s="3" t="n">
-        <v>3.4</v>
+        <v>3</v>
       </c>
       <c r="P13" s="3" t="n">
         <v>3.4</v>
@@ -1163,7 +1163,7 @@
     </row>
     <row r="14">
       <c r="A14" s="3" t="n">
-        <v>32</v>
+        <v>22</v>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
@@ -1171,207 +1171,207 @@
         </is>
       </c>
       <c r="C14" s="3" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="D14" s="3" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="E14" s="3" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="F14" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="G14" s="3" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="H14" s="3" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="I14" s="3" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="J14" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="K14" s="3" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="L14" s="3" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="M14" s="3" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="N14" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="D14" s="3" t="n">
-        <v>4.25</v>
-      </c>
-      <c r="E14" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="F14" s="3" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="G14" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="H14" s="3" t="n">
-        <v>2.25</v>
-      </c>
-      <c r="I14" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="J14" s="3" t="n">
-        <v>1.6</v>
-      </c>
-      <c r="K14" s="3" t="n">
-        <v>4.4</v>
-      </c>
-      <c r="L14" s="3" t="n">
-        <v>1.6</v>
-      </c>
-      <c r="M14" s="3" t="n">
-        <v>4.8</v>
-      </c>
-      <c r="N14" s="3" t="n">
-        <v>2.6</v>
-      </c>
       <c r="O14" s="3" t="n">
-        <v>5</v>
+        <v>3.6</v>
       </c>
       <c r="P14" s="3" t="n">
-        <v>1.2</v>
+        <v>3.2</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="n">
-        <v>3</v>
+        <v>27</v>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>CS1</t>
+          <t>CS0</t>
         </is>
       </c>
       <c r="C15" s="3" t="n">
-        <v>3.5</v>
+        <v>3</v>
       </c>
       <c r="D15" s="3" t="n">
         <v>3</v>
       </c>
       <c r="E15" s="3" t="n">
-        <v>4.5</v>
+        <v>4</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>3.25</v>
+        <v>4</v>
       </c>
       <c r="H15" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I15" s="3" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="J15" s="3" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="K15" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="J15" s="3" t="n">
-        <v>2.4</v>
-      </c>
-      <c r="K15" s="3" t="n">
-        <v>3.6</v>
-      </c>
       <c r="L15" s="3" t="n">
-        <v>3.6</v>
+        <v>4.4</v>
       </c>
       <c r="M15" s="3" t="n">
-        <v>1.6</v>
+        <v>4.4</v>
       </c>
       <c r="N15" s="3" t="n">
-        <v>2</v>
+        <v>3.2</v>
       </c>
       <c r="O15" s="3" t="n">
-        <v>4</v>
+        <v>3.4</v>
       </c>
       <c r="P15" s="3" t="n">
-        <v>3.8</v>
+        <v>3.4</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="n">
-        <v>8</v>
+        <v>32</v>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>CS1</t>
+          <t>CS0</t>
         </is>
       </c>
       <c r="C16" s="3" t="n">
-        <v>3.25</v>
+        <v>4</v>
       </c>
       <c r="D16" s="3" t="n">
+        <v>4.25</v>
+      </c>
+      <c r="E16" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="F16" s="3" t="n">
         <v>2.5</v>
       </c>
-      <c r="E16" s="3" t="n">
-        <v>2.75</v>
-      </c>
-      <c r="F16" s="3" t="n">
-        <v>2.75</v>
-      </c>
       <c r="G16" s="3" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H16" s="3" t="n">
-        <v>2</v>
+        <v>2.25</v>
       </c>
       <c r="I16" s="3" t="n">
-        <v>1.6</v>
+        <v>5</v>
       </c>
       <c r="J16" s="3" t="n">
         <v>1.6</v>
       </c>
       <c r="K16" s="3" t="n">
-        <v>1.8</v>
+        <v>4.4</v>
       </c>
       <c r="L16" s="3" t="n">
-        <v>2</v>
+        <v>1.6</v>
       </c>
       <c r="M16" s="3" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="N16" s="3" t="n">
         <v>2.6</v>
       </c>
-      <c r="N16" s="3" t="n">
-        <v>2.4</v>
-      </c>
       <c r="O16" s="3" t="n">
-        <v>2.8</v>
+        <v>5</v>
       </c>
       <c r="P16" s="3" t="n">
-        <v>2.6</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="n">
-        <v>13</v>
+        <v>37</v>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>CS1</t>
+          <t>CS0</t>
         </is>
       </c>
       <c r="C17" s="3" t="n">
         <v>2.75</v>
       </c>
       <c r="D17" s="3" t="n">
-        <v>3</v>
+        <v>2.75</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>2.5</v>
+        <v>3</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>3.5</v>
+        <v>1.5</v>
       </c>
       <c r="G17" s="3" t="n">
-        <v>2.75</v>
+        <v>3.25</v>
       </c>
       <c r="H17" s="3" t="n">
-        <v>2.75</v>
+        <v>1.25</v>
       </c>
       <c r="I17" s="3" t="n">
-        <v>3.2</v>
+        <v>4.6</v>
       </c>
       <c r="J17" s="3" t="n">
-        <v>3.4</v>
+        <v>1.8</v>
       </c>
       <c r="K17" s="3" t="n">
-        <v>2.6</v>
+        <v>4.4</v>
       </c>
       <c r="L17" s="3" t="n">
-        <v>3.4</v>
+        <v>2.2</v>
       </c>
       <c r="M17" s="3" t="n">
-        <v>2.4</v>
+        <v>2.8</v>
       </c>
       <c r="N17" s="3" t="n">
-        <v>3.2</v>
+        <v>1.6</v>
       </c>
       <c r="O17" s="3" t="n">
-        <v>3.4</v>
+        <v>2.8</v>
       </c>
       <c r="P17" s="3" t="n">
-        <v>3.4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="n">
-        <v>18</v>
+        <v>3</v>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
@@ -1379,51 +1379,51 @@
         </is>
       </c>
       <c r="C18" s="3" t="n">
-        <v>1</v>
+        <v>3.5</v>
       </c>
       <c r="D18" s="3" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E18" s="3" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="F18" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="G18" s="3" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="H18" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="I18" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="F18" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="G18" s="3" t="n">
-        <v>2.75</v>
-      </c>
-      <c r="H18" s="3" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="I18" s="3" t="n">
+      <c r="J18" s="3" t="n">
         <v>2.4</v>
       </c>
-      <c r="J18" s="3" t="n">
+      <c r="K18" s="3" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="L18" s="3" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="M18" s="3" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="N18" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="K18" s="3" t="n">
-        <v>2.6</v>
-      </c>
-      <c r="L18" s="3" t="n">
-        <v>2.2</v>
-      </c>
-      <c r="M18" s="3" t="n">
-        <v>2.6</v>
-      </c>
-      <c r="N18" s="3" t="n">
-        <v>2.6</v>
-      </c>
       <c r="O18" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="P18" s="3" t="n">
-        <v>2.8</v>
+        <v>3.8</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="n">
-        <v>23</v>
+        <v>8</v>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
@@ -1431,51 +1431,51 @@
         </is>
       </c>
       <c r="C19" s="3" t="n">
-        <v>3.5</v>
+        <v>3.25</v>
       </c>
       <c r="D19" s="3" t="n">
-        <v>3.75</v>
+        <v>2.5</v>
       </c>
       <c r="E19" s="3" t="n">
-        <v>4.75</v>
+        <v>2.75</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>4.75</v>
+        <v>2.75</v>
       </c>
       <c r="G19" s="3" t="n">
-        <v>4.5</v>
+        <v>3</v>
       </c>
       <c r="H19" s="3" t="n">
-        <v>4.5</v>
+        <v>2</v>
       </c>
       <c r="I19" s="3" t="n">
-        <v>3.2</v>
+        <v>1.6</v>
       </c>
       <c r="J19" s="3" t="n">
-        <v>3</v>
+        <v>1.6</v>
       </c>
       <c r="K19" s="3" t="n">
-        <v>3</v>
+        <v>1.8</v>
       </c>
       <c r="L19" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="M19" s="3" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="N19" s="3" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="O19" s="3" t="n">
         <v>2.8</v>
       </c>
-      <c r="M19" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="N19" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="O19" s="3" t="n">
-        <v>3</v>
-      </c>
       <c r="P19" s="3" t="n">
-        <v>3</v>
+        <v>2.6</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="n">
-        <v>28</v>
+        <v>13</v>
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
@@ -1483,51 +1483,51 @@
         </is>
       </c>
       <c r="C20" s="3" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="D20" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E20" s="3" t="n">
         <v>2.5</v>
       </c>
-      <c r="D20" s="3" t="n">
-        <v>1.75</v>
-      </c>
-      <c r="E20" s="3" t="n">
-        <v>4.75</v>
-      </c>
       <c r="F20" s="3" t="n">
-        <v>4</v>
+        <v>3.5</v>
       </c>
       <c r="G20" s="3" t="n">
-        <v>4.5</v>
+        <v>2.75</v>
       </c>
       <c r="H20" s="3" t="n">
-        <v>4.5</v>
+        <v>2.75</v>
       </c>
       <c r="I20" s="3" t="n">
-        <v>3</v>
+        <v>3.2</v>
       </c>
       <c r="J20" s="3" t="n">
-        <v>3.6</v>
+        <v>3.4</v>
       </c>
       <c r="K20" s="3" t="n">
-        <v>3.8</v>
+        <v>2.6</v>
       </c>
       <c r="L20" s="3" t="n">
-        <v>4.2</v>
+        <v>3.4</v>
       </c>
       <c r="M20" s="3" t="n">
-        <v>2.2</v>
+        <v>2.4</v>
       </c>
       <c r="N20" s="3" t="n">
-        <v>1.8</v>
+        <v>3.2</v>
       </c>
       <c r="O20" s="3" t="n">
-        <v>3.8</v>
+        <v>3.4</v>
       </c>
       <c r="P20" s="3" t="n">
-        <v>3.6</v>
+        <v>3.4</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="n">
-        <v>33</v>
+        <v>18</v>
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
@@ -1535,215 +1535,215 @@
         </is>
       </c>
       <c r="C21" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D21" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E21" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="D21" s="3" t="n">
-        <v>3.75</v>
-      </c>
-      <c r="E21" s="3" t="n">
-        <v>5</v>
-      </c>
       <c r="F21" s="3" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>4.5</v>
+        <v>2.75</v>
       </c>
       <c r="H21" s="3" t="n">
-        <v>4.5</v>
+        <v>2.5</v>
       </c>
       <c r="I21" s="3" t="n">
-        <v>4.6</v>
+        <v>2.4</v>
       </c>
       <c r="J21" s="3" t="n">
-        <v>4.4</v>
+        <v>2</v>
       </c>
       <c r="K21" s="3" t="n">
-        <v>4.6</v>
+        <v>2.6</v>
       </c>
       <c r="L21" s="3" t="n">
-        <v>4.4</v>
+        <v>2.2</v>
       </c>
       <c r="M21" s="3" t="n">
-        <v>3.8</v>
+        <v>2.6</v>
       </c>
       <c r="N21" s="3" t="n">
-        <v>4</v>
+        <v>2.6</v>
       </c>
       <c r="O21" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="P21" s="3" t="n">
         <v>2.8</v>
-      </c>
-      <c r="P21" s="3" t="n">
-        <v>2.4</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="n">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>CI</t>
+          <t>CS1</t>
         </is>
       </c>
       <c r="C22" s="3" t="n">
-        <v>2.75</v>
+        <v>3.5</v>
       </c>
       <c r="D22" s="3" t="n">
-        <v>2</v>
+        <v>3.75</v>
       </c>
       <c r="E22" s="3" t="n">
-        <v>3.75</v>
+        <v>4.75</v>
       </c>
       <c r="F22" s="3" t="n">
-        <v>3.5</v>
+        <v>4.75</v>
       </c>
       <c r="G22" s="3" t="n">
-        <v>4</v>
+        <v>4.5</v>
       </c>
       <c r="H22" s="3" t="n">
-        <v>5</v>
+        <v>4.5</v>
       </c>
       <c r="I22" s="3" t="n">
-        <v>4.4</v>
+        <v>3.2</v>
       </c>
       <c r="J22" s="3" t="n">
-        <v>3.2</v>
+        <v>3</v>
       </c>
       <c r="K22" s="3" t="n">
-        <v>4.2</v>
+        <v>3</v>
       </c>
       <c r="L22" s="3" t="n">
         <v>2.8</v>
       </c>
       <c r="M22" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N22" s="3" t="n">
-        <v>2.2</v>
+        <v>4</v>
       </c>
       <c r="O22" s="3" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="P22" s="3" t="n">
-        <v>3.6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="n">
-        <v>9</v>
+        <v>28</v>
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>CI</t>
+          <t>CS1</t>
         </is>
       </c>
       <c r="C23" s="3" t="n">
         <v>2.5</v>
       </c>
       <c r="D23" s="3" t="n">
-        <v>2.5</v>
+        <v>1.75</v>
       </c>
       <c r="E23" s="3" t="n">
+        <v>4.75</v>
+      </c>
+      <c r="F23" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="F23" s="3" t="n">
-        <v>1.5</v>
-      </c>
       <c r="G23" s="3" t="n">
-        <v>3.5</v>
+        <v>4.5</v>
       </c>
       <c r="H23" s="3" t="n">
-        <v>1</v>
+        <v>4.5</v>
       </c>
       <c r="I23" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="J23" s="3" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="K23" s="3" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="L23" s="3" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="M23" s="3" t="n">
         <v>2.2</v>
-      </c>
-      <c r="J23" s="3" t="n">
-        <v>2.8</v>
-      </c>
-      <c r="K23" s="3" t="n">
-        <v>2.8</v>
-      </c>
-      <c r="L23" s="3" t="n">
-        <v>2.4</v>
-      </c>
-      <c r="M23" s="3" t="n">
-        <v>3.2</v>
       </c>
       <c r="N23" s="3" t="n">
         <v>1.8</v>
       </c>
       <c r="O23" s="3" t="n">
-        <v>3.4</v>
+        <v>3.8</v>
       </c>
       <c r="P23" s="3" t="n">
-        <v>2.4</v>
+        <v>3.6</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="n">
-        <v>14</v>
+        <v>33</v>
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>CI</t>
+          <t>CS1</t>
         </is>
       </c>
       <c r="C24" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D24" s="3" t="n">
-        <v>3.25</v>
+        <v>3.75</v>
       </c>
       <c r="E24" s="3" t="n">
-        <v>3.5</v>
+        <v>5</v>
       </c>
       <c r="F24" s="3" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G24" s="3" t="n">
-        <v>3.25</v>
+        <v>4.5</v>
       </c>
       <c r="H24" s="3" t="n">
-        <v>3</v>
+        <v>4.5</v>
       </c>
       <c r="I24" s="3" t="n">
-        <v>3.4</v>
+        <v>4.6</v>
       </c>
       <c r="J24" s="3" t="n">
-        <v>2.2</v>
+        <v>4.4</v>
       </c>
       <c r="K24" s="3" t="n">
-        <v>3.6</v>
+        <v>4.6</v>
       </c>
       <c r="L24" s="3" t="n">
-        <v>2</v>
+        <v>4.4</v>
       </c>
       <c r="M24" s="3" t="n">
         <v>3.8</v>
       </c>
       <c r="N24" s="3" t="n">
-        <v>2.8</v>
+        <v>4</v>
       </c>
       <c r="O24" s="3" t="n">
         <v>2.8</v>
       </c>
       <c r="P24" s="3" t="n">
-        <v>1.8</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="n">
-        <v>19</v>
+        <v>38</v>
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>CI</t>
+          <t>CS1</t>
         </is>
       </c>
       <c r="C25" s="3" t="n">
-        <v>2.5</v>
+        <v>2.25</v>
       </c>
       <c r="D25" s="3" t="n">
         <v>2.5</v>
@@ -1752,25 +1752,25 @@
         <v>3.75</v>
       </c>
       <c r="F25" s="3" t="n">
-        <v>1</v>
+        <v>3.75</v>
       </c>
       <c r="G25" s="3" t="n">
-        <v>3.5</v>
+        <v>4</v>
       </c>
       <c r="H25" s="3" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I25" s="3" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="J25" s="3" t="n">
         <v>2.6</v>
       </c>
-      <c r="J25" s="3" t="n">
-        <v>1.8</v>
-      </c>
       <c r="K25" s="3" t="n">
-        <v>2.4</v>
+        <v>4.4</v>
       </c>
       <c r="L25" s="3" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="M25" s="3" t="n">
         <v>2.8</v>
@@ -1779,15 +1779,15 @@
         <v>2.8</v>
       </c>
       <c r="O25" s="3" t="n">
-        <v>1.6</v>
+        <v>3.2</v>
       </c>
       <c r="P25" s="3" t="n">
-        <v>1.4</v>
+        <v>3.4</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="n">
-        <v>24</v>
+        <v>4</v>
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
@@ -1798,48 +1798,48 @@
         <v>2.75</v>
       </c>
       <c r="D26" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E26" s="3" t="n">
         <v>3.75</v>
       </c>
-      <c r="E26" s="3" t="n">
-        <v>3</v>
-      </c>
       <c r="F26" s="3" t="n">
-        <v>1.25</v>
+        <v>3.5</v>
       </c>
       <c r="G26" s="3" t="n">
-        <v>3.25</v>
+        <v>4</v>
       </c>
       <c r="H26" s="3" t="n">
-        <v>2.75</v>
+        <v>5</v>
       </c>
       <c r="I26" s="3" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="J26" s="3" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="K26" s="3" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="L26" s="3" t="n">
         <v>2.8</v>
       </c>
-      <c r="J26" s="3" t="n">
-        <v>1.8</v>
-      </c>
-      <c r="K26" s="3" t="n">
+      <c r="M26" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="N26" s="3" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="O26" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="P26" s="3" t="n">
         <v>3.6</v>
-      </c>
-      <c r="L26" s="3" t="n">
-        <v>1.8</v>
-      </c>
-      <c r="M26" s="3" t="n">
-        <v>3.4</v>
-      </c>
-      <c r="N26" s="3" t="n">
-        <v>3.2</v>
-      </c>
-      <c r="O26" s="3" t="n">
-        <v>2.4</v>
-      </c>
-      <c r="P26" s="3" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="n">
-        <v>29</v>
+        <v>9</v>
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
@@ -1847,51 +1847,51 @@
         </is>
       </c>
       <c r="C27" s="3" t="n">
-        <v>2.75</v>
+        <v>2.5</v>
       </c>
       <c r="D27" s="3" t="n">
-        <v>2.25</v>
+        <v>2.5</v>
       </c>
       <c r="E27" s="3" t="n">
-        <v>2.75</v>
+        <v>4</v>
       </c>
       <c r="F27" s="3" t="n">
         <v>1.5</v>
       </c>
       <c r="G27" s="3" t="n">
-        <v>2.5</v>
+        <v>3.5</v>
       </c>
       <c r="H27" s="3" t="n">
         <v>1</v>
       </c>
       <c r="I27" s="3" t="n">
-        <v>2</v>
+        <v>2.2</v>
       </c>
       <c r="J27" s="3" t="n">
-        <v>2</v>
+        <v>2.8</v>
       </c>
       <c r="K27" s="3" t="n">
-        <v>2.6</v>
+        <v>2.8</v>
       </c>
       <c r="L27" s="3" t="n">
-        <v>2</v>
+        <v>2.4</v>
       </c>
       <c r="M27" s="3" t="n">
-        <v>2.6</v>
+        <v>3.2</v>
       </c>
       <c r="N27" s="3" t="n">
-        <v>2.2</v>
+        <v>1.8</v>
       </c>
       <c r="O27" s="3" t="n">
-        <v>2.2</v>
+        <v>3.4</v>
       </c>
       <c r="P27" s="3" t="n">
-        <v>2</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="3" t="n">
-        <v>34</v>
+        <v>14</v>
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
@@ -1899,263 +1899,263 @@
         </is>
       </c>
       <c r="C28" s="3" t="n">
-        <v>2.5</v>
+        <v>3</v>
       </c>
       <c r="D28" s="3" t="n">
-        <v>2</v>
+        <v>3.25</v>
       </c>
       <c r="E28" s="3" t="n">
         <v>3.5</v>
       </c>
       <c r="F28" s="3" t="n">
-        <v>3.5</v>
+        <v>3</v>
       </c>
       <c r="G28" s="3" t="n">
-        <v>3</v>
+        <v>3.25</v>
       </c>
       <c r="H28" s="3" t="n">
-        <v>2.75</v>
+        <v>3</v>
       </c>
       <c r="I28" s="3" t="n">
-        <v>2.6</v>
+        <v>3.4</v>
       </c>
       <c r="J28" s="3" t="n">
-        <v>3.4</v>
+        <v>2.2</v>
       </c>
       <c r="K28" s="3" t="n">
-        <v>4</v>
+        <v>3.6</v>
       </c>
       <c r="L28" s="3" t="n">
-        <v>2.4</v>
+        <v>2</v>
       </c>
       <c r="M28" s="3" t="n">
         <v>3.8</v>
       </c>
       <c r="N28" s="3" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="O28" s="3" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="P28" s="3" t="n">
         <v>1.8</v>
-      </c>
-      <c r="O28" s="3" t="n">
-        <v>1.6</v>
-      </c>
-      <c r="P28" s="3" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="3" t="n">
-        <v>5</v>
+        <v>19</v>
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>II</t>
+          <t>CI</t>
         </is>
       </c>
       <c r="C29" s="3" t="n">
-        <v>2.75</v>
+        <v>2.5</v>
       </c>
       <c r="D29" s="3" t="n">
-        <v>2.75</v>
+        <v>2.5</v>
       </c>
       <c r="E29" s="3" t="n">
-        <v>4</v>
+        <v>3.75</v>
       </c>
       <c r="F29" s="3" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G29" s="3" t="n">
-        <v>1.75</v>
+        <v>3.5</v>
       </c>
       <c r="H29" s="3" t="n">
-        <v>1.5</v>
+        <v>1</v>
       </c>
       <c r="I29" s="3" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="J29" s="3" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="K29" s="3" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="L29" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="M29" s="3" t="n">
         <v>2.8</v>
       </c>
-      <c r="J29" s="3" t="n">
+      <c r="N29" s="3" t="n">
         <v>2.8</v>
       </c>
-      <c r="K29" s="3" t="n">
-        <v>3.2</v>
-      </c>
-      <c r="L29" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="M29" s="3" t="n">
-        <v>3.8</v>
-      </c>
-      <c r="N29" s="3" t="n">
-        <v>3</v>
-      </c>
       <c r="O29" s="3" t="n">
-        <v>2.6</v>
+        <v>1.6</v>
       </c>
       <c r="P29" s="3" t="n">
-        <v>2.2</v>
+        <v>1.4</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="3" t="n">
-        <v>10</v>
+        <v>24</v>
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>II</t>
+          <t>CI</t>
         </is>
       </c>
       <c r="C30" s="3" t="n">
-        <v>2</v>
+        <v>2.75</v>
       </c>
       <c r="D30" s="3" t="n">
-        <v>1.25</v>
+        <v>3.75</v>
       </c>
       <c r="E30" s="3" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F30" s="3" t="n">
         <v>1.25</v>
       </c>
       <c r="G30" s="3" t="n">
-        <v>1.25</v>
+        <v>3.25</v>
       </c>
       <c r="H30" s="3" t="n">
-        <v>1.5</v>
+        <v>2.75</v>
       </c>
       <c r="I30" s="3" t="n">
-        <v>2.2</v>
+        <v>2.8</v>
       </c>
       <c r="J30" s="3" t="n">
         <v>1.8</v>
       </c>
       <c r="K30" s="3" t="n">
-        <v>1.6</v>
+        <v>3.6</v>
       </c>
       <c r="L30" s="3" t="n">
-        <v>1.4</v>
+        <v>1.8</v>
       </c>
       <c r="M30" s="3" t="n">
-        <v>1.6</v>
+        <v>3.4</v>
       </c>
       <c r="N30" s="3" t="n">
-        <v>1.8</v>
+        <v>3.2</v>
       </c>
       <c r="O30" s="3" t="n">
-        <v>1.2</v>
+        <v>2.4</v>
       </c>
       <c r="P30" s="3" t="n">
-        <v>1.6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="3" t="n">
-        <v>15</v>
+        <v>29</v>
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>II</t>
+          <t>CI</t>
         </is>
       </c>
       <c r="C31" s="3" t="n">
-        <v>1.75</v>
+        <v>2.75</v>
       </c>
       <c r="D31" s="3" t="n">
-        <v>1.75</v>
+        <v>2.25</v>
       </c>
       <c r="E31" s="3" t="n">
-        <v>1</v>
+        <v>2.75</v>
       </c>
       <c r="F31" s="3" t="n">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="G31" s="3" t="n">
-        <v>1.75</v>
+        <v>2.5</v>
       </c>
       <c r="H31" s="3" t="n">
-        <v>1.5</v>
+        <v>1</v>
       </c>
       <c r="I31" s="3" t="n">
-        <v>1.4</v>
+        <v>2</v>
       </c>
       <c r="J31" s="3" t="n">
-        <v>1.2</v>
+        <v>2</v>
       </c>
       <c r="K31" s="3" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="L31" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="L31" s="3" t="n">
-        <v>1.6</v>
-      </c>
       <c r="M31" s="3" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="N31" s="3" t="n">
         <v>2.2</v>
       </c>
-      <c r="N31" s="3" t="n">
+      <c r="O31" s="3" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="P31" s="3" t="n">
         <v>2</v>
-      </c>
-      <c r="O31" s="3" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="P31" s="3" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="3" t="n">
-        <v>20</v>
+        <v>34</v>
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>II</t>
+          <t>CI</t>
         </is>
       </c>
       <c r="C32" s="3" t="n">
-        <v>3</v>
+        <v>2.5</v>
       </c>
       <c r="D32" s="3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E32" s="3" t="n">
-        <v>3.25</v>
+        <v>3.5</v>
       </c>
       <c r="F32" s="3" t="n">
-        <v>3</v>
+        <v>3.5</v>
       </c>
       <c r="G32" s="3" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H32" s="3" t="n">
-        <v>2</v>
+        <v>2.75</v>
       </c>
       <c r="I32" s="3" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="J32" s="3" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="K32" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="L32" s="3" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="M32" s="3" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="N32" s="3" t="n">
         <v>1.8</v>
       </c>
-      <c r="J32" s="3" t="n">
-        <v>2.6</v>
-      </c>
-      <c r="K32" s="3" t="n">
-        <v>2.8</v>
-      </c>
-      <c r="L32" s="3" t="n">
-        <v>3.2</v>
-      </c>
-      <c r="M32" s="3" t="n">
-        <v>2.8</v>
-      </c>
-      <c r="N32" s="3" t="n">
-        <v>2.4</v>
-      </c>
       <c r="O32" s="3" t="n">
-        <v>2.6</v>
+        <v>1.6</v>
       </c>
       <c r="P32" s="3" t="n">
-        <v>2.8</v>
+        <v>1</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="3" t="n">
-        <v>25</v>
+        <v>39</v>
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>II</t>
+          <t>CI</t>
         </is>
       </c>
       <c r="C33" s="3" t="n">
@@ -2165,45 +2165,45 @@
         <v>2</v>
       </c>
       <c r="E33" s="3" t="n">
-        <v>2.5</v>
+        <v>3.5</v>
       </c>
       <c r="F33" s="3" t="n">
-        <v>2.25</v>
+        <v>3</v>
       </c>
       <c r="G33" s="3" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H33" s="3" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I33" s="3" t="n">
         <v>1.8</v>
       </c>
       <c r="J33" s="3" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="K33" s="3" t="n">
         <v>2.2</v>
       </c>
-      <c r="K33" s="3" t="n">
+      <c r="L33" s="3" t="n">
         <v>2.8</v>
       </c>
-      <c r="L33" s="3" t="n">
-        <v>2.2</v>
-      </c>
       <c r="M33" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="N33" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="O33" s="3" t="n">
         <v>1.8</v>
       </c>
-      <c r="N33" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="O33" s="3" t="n">
-        <v>3.4</v>
-      </c>
       <c r="P33" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="3" t="n">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
@@ -2211,43 +2211,43 @@
         </is>
       </c>
       <c r="C34" s="3" t="n">
-        <v>3.75</v>
+        <v>2.75</v>
       </c>
       <c r="D34" s="3" t="n">
-        <v>3.75</v>
+        <v>2.75</v>
       </c>
       <c r="E34" s="3" t="n">
         <v>4</v>
       </c>
       <c r="F34" s="3" t="n">
-        <v>3.75</v>
+        <v>4</v>
       </c>
       <c r="G34" s="3" t="n">
-        <v>3.5</v>
+        <v>1.75</v>
       </c>
       <c r="H34" s="3" t="n">
-        <v>3</v>
+        <v>1.5</v>
       </c>
       <c r="I34" s="3" t="n">
         <v>2.8</v>
       </c>
       <c r="J34" s="3" t="n">
-        <v>3.4</v>
+        <v>2.8</v>
       </c>
       <c r="K34" s="3" t="n">
-        <v>3.4</v>
+        <v>3.2</v>
       </c>
       <c r="L34" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="M34" s="3" t="n">
         <v>3.8</v>
       </c>
-      <c r="M34" s="3" t="n">
-        <v>2.8</v>
-      </c>
       <c r="N34" s="3" t="n">
-        <v>4.2</v>
+        <v>3</v>
       </c>
       <c r="O34" s="3" t="n">
-        <v>2</v>
+        <v>2.6</v>
       </c>
       <c r="P34" s="3" t="n">
         <v>2.2</v>
@@ -2255,7 +2255,7 @@
     </row>
     <row r="35">
       <c r="A35" s="3" t="n">
-        <v>35</v>
+        <v>10</v>
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
@@ -2263,46 +2263,358 @@
         </is>
       </c>
       <c r="C35" s="3" t="n">
-        <v>2.5</v>
+        <v>2</v>
       </c>
       <c r="D35" s="3" t="n">
-        <v>2</v>
+        <v>1.25</v>
       </c>
       <c r="E35" s="3" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F35" s="3" t="n">
-        <v>3.25</v>
+        <v>1.25</v>
       </c>
       <c r="G35" s="3" t="n">
-        <v>1</v>
+        <v>1.25</v>
       </c>
       <c r="H35" s="3" t="n">
         <v>1.5</v>
       </c>
       <c r="I35" s="3" t="n">
-        <v>2</v>
+        <v>2.2</v>
       </c>
       <c r="J35" s="3" t="n">
-        <v>1</v>
+        <v>1.8</v>
       </c>
       <c r="K35" s="3" t="n">
         <v>1.6</v>
       </c>
       <c r="L35" s="3" t="n">
-        <v>1</v>
+        <v>1.4</v>
       </c>
       <c r="M35" s="3" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="N35" s="3" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="O35" s="3" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="P35" s="3" t="n">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>II</t>
+        </is>
+      </c>
+      <c r="C36" s="3" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="D36" s="3" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="E36" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F36" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G36" s="3" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="H36" s="3" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="I36" s="3" t="n">
         <v>1.4</v>
       </c>
-      <c r="N35" s="3" t="n">
+      <c r="J36" s="3" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="K36" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="L36" s="3" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="M36" s="3" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="N36" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="O36" s="3" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="P36" s="3" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="B37" s="3" t="inlineStr">
+        <is>
+          <t>II</t>
+        </is>
+      </c>
+      <c r="C37" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="D37" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E37" s="3" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="F37" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="G37" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="H37" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="I37" s="3" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="J37" s="3" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="K37" s="3" t="n">
         <v>2.8</v>
       </c>
-      <c r="O35" s="3" t="n">
+      <c r="L37" s="3" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="M37" s="3" t="n">
         <v>2.8</v>
       </c>
-      <c r="P35" s="3" t="n">
+      <c r="N37" s="3" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="O37" s="3" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="P37" s="3" t="n">
+        <v>2.8</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="3" t="n">
+        <v>25</v>
+      </c>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>II</t>
+        </is>
+      </c>
+      <c r="C38" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D38" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E38" s="3" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F38" s="3" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="G38" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="H38" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="I38" s="3" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="J38" s="3" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="K38" s="3" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="L38" s="3" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="M38" s="3" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="N38" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="O38" s="3" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="P38" s="3" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="B39" s="3" t="inlineStr">
+        <is>
+          <t>II</t>
+        </is>
+      </c>
+      <c r="C39" s="3" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="D39" s="3" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="E39" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="F39" s="3" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="G39" s="3" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="H39" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="I39" s="3" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="J39" s="3" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="K39" s="3" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="L39" s="3" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="M39" s="3" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="N39" s="3" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="O39" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="P39" s="3" t="n">
+        <v>2.2</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="3" t="n">
+        <v>35</v>
+      </c>
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>II</t>
+        </is>
+      </c>
+      <c r="C40" s="3" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="D40" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E40" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="F40" s="3" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="G40" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="H40" s="3" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="I40" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="J40" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="K40" s="3" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="L40" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="M40" s="3" t="n">
         <v>1.4</v>
+      </c>
+      <c r="N40" s="3" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="O40" s="3" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="P40" s="3" t="n">
+        <v>1.4</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="3" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" s="3" t="inlineStr">
+        <is>
+          <t>II</t>
+        </is>
+      </c>
+      <c r="C41" s="3" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="D41" s="3" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="E41" s="3" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="F41" s="3" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="G41" s="3" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="H41" s="3" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="I41" s="3" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="J41" s="3" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="K41" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="L41" s="3" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="M41" s="3" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="N41" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="O41" s="3" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="P41" s="3" t="n">
+        <v>1.6</v>
       </c>
     </row>
   </sheetData>
@@ -2376,10 +2688,10 @@
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>0.437986860330652</v>
+        <v>0.979238682212762</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>0.780072857046435</v>
+        <v>0.431403539796531</v>
       </c>
       <c r="F2" s="3" t="b">
         <v>0</v>
@@ -2402,10 +2714,10 @@
         </is>
       </c>
       <c r="D3" s="3" t="n">
-        <v>1.608094377369087</v>
+        <v>1.338038719612804</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>0.1989075188872209</v>
+        <v>0.2753019020930046</v>
       </c>
       <c r="F3" s="3" t="b">
         <v>0</v>
@@ -2428,10 +2740,10 @@
         </is>
       </c>
       <c r="D4" s="3" t="n">
-        <v>7.55817881835324</v>
+        <v>9.205523451845574</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>0.1091710477856081</v>
+        <v>0.05616272016762326</v>
       </c>
       <c r="F4" s="3" t="b">
         <v>0</v>
@@ -2454,10 +2766,10 @@
         </is>
       </c>
       <c r="D5" s="3" t="n">
-        <v>7.310142790625485</v>
+        <v>8.461582456999572</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>0.1203785224047728</v>
+        <v>0.07606031193307826</v>
       </c>
       <c r="F5" s="3" t="b">
         <v>0</v>
@@ -2480,10 +2792,10 @@
         </is>
       </c>
       <c r="D6" s="3" t="n">
-        <v>14.91758963044678</v>
+        <v>17.39210567666436</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>0.004875229451904635</v>
+        <v>0.001621612978210302</v>
       </c>
       <c r="F6" s="3" t="b">
         <v>1</v>
@@ -2506,10 +2818,10 @@
         </is>
       </c>
       <c r="D7" s="3" t="n">
-        <v>10.16852419942179</v>
+        <v>12.0904833736041</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>0.03768260691296652</v>
+        <v>0.01669093976383364</v>
       </c>
       <c r="F7" s="3" t="b">
         <v>1</v>
@@ -2540,13 +2852,13 @@
         </is>
       </c>
       <c r="D9" s="3" t="n">
-        <v>-2.517439175034821</v>
+        <v>-0.25</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>0.04544403991949149</v>
+        <v>0.8088874454935351</v>
       </c>
       <c r="F9" s="3" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
@@ -2566,10 +2878,10 @@
         </is>
       </c>
       <c r="D10" s="3" t="n">
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>0.25</v>
+        <v>0.1875</v>
       </c>
       <c r="F10" s="3" t="b">
         <v>0</v>
@@ -2592,10 +2904,10 @@
         </is>
       </c>
       <c r="D11" s="3" t="n">
-        <v>-1.111437860452423</v>
+        <v>-1.276939015148195</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>0.3089213661430785</v>
+        <v>0.2374378627385179</v>
       </c>
       <c r="F11" s="3" t="b">
         <v>0</v>
@@ -2652,10 +2964,10 @@
         </is>
       </c>
       <c r="D14" s="3" t="n">
-        <v>1.242259987499883</v>
+        <v>1.692228224453299</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>0.2692267472099367</v>
+        <v>0.1415500090567489</v>
       </c>
       <c r="F14" s="3" t="b">
         <v>0</v>
@@ -2678,10 +2990,10 @@
         </is>
       </c>
       <c r="D15" s="3" t="n">
-        <v>1.706574098530288</v>
+        <v>2.208193696890079</v>
       </c>
       <c r="E15" s="3" t="n">
-        <v>0.1486119507797838</v>
+        <v>0.06931549051135975</v>
       </c>
       <c r="F15" s="3" t="b">
         <v>0</v>
@@ -2712,10 +3024,10 @@
         </is>
       </c>
       <c r="D17" s="3" t="n">
-        <v>1.527525231651947</v>
+        <v>1.210419877178893</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>0.1774888324162401</v>
+        <v>0.2653980394260696</v>
       </c>
       <c r="F17" s="3" t="b">
         <v>0</v>
@@ -2738,10 +3050,10 @@
         </is>
       </c>
       <c r="D18" s="3" t="n">
-        <v>1.030114251517296</v>
+        <v>1.029472235716996</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>0.3426799101911869</v>
+        <v>0.3375098903355412</v>
       </c>
       <c r="F18" s="3" t="b">
         <v>0</v>
@@ -2767,7 +3079,7 @@
         <v>0</v>
       </c>
       <c r="E19" s="3" t="n">
-        <v>0.25</v>
+        <v>0.125</v>
       </c>
       <c r="F19" s="3" t="b">
         <v>0</v>
@@ -2798,10 +3110,10 @@
         </is>
       </c>
       <c r="D21" s="3" t="n">
-        <v>0.3202563076101743</v>
+        <v>0.3232299675777271</v>
       </c>
       <c r="E21" s="3" t="n">
-        <v>0.7596334165649292</v>
+        <v>0.7559627503969001</v>
       </c>
       <c r="F21" s="3" t="b">
         <v>0</v>
@@ -2824,10 +3136,10 @@
         </is>
       </c>
       <c r="D22" s="3" t="n">
-        <v>3.109926332092897</v>
+        <v>3.198557367121814</v>
       </c>
       <c r="E22" s="3" t="n">
-        <v>0.0208508042624513</v>
+        <v>0.015096034879553</v>
       </c>
       <c r="F22" s="3" t="b">
         <v>1</v>
@@ -2850,10 +3162,10 @@
         </is>
       </c>
       <c r="D23" s="3" t="n">
-        <v>1.894566053473315</v>
+        <v>1.846407837401394</v>
       </c>
       <c r="E23" s="3" t="n">
-        <v>0.1069727465609034</v>
+        <v>0.1073313153411767</v>
       </c>
       <c r="F23" s="3" t="b">
         <v>0</v>
@@ -2910,10 +3222,10 @@
         </is>
       </c>
       <c r="D26" s="3" t="n">
-        <v>0.4200840252084029</v>
+        <v>-0.3139929128113796</v>
       </c>
       <c r="E26" s="3" t="n">
-        <v>0.6890522264439654</v>
+        <v>0.7626770646286338</v>
       </c>
       <c r="F26" s="3" t="b">
         <v>0</v>
@@ -2936,10 +3248,10 @@
         </is>
       </c>
       <c r="D27" s="3" t="n">
-        <v>-0.5477225575051661</v>
+        <v>-0.5516772843673705</v>
       </c>
       <c r="E27" s="3" t="n">
-        <v>0.6036450565101363</v>
+        <v>0.5983311559987459</v>
       </c>
       <c r="F27" s="3" t="b">
         <v>0</v>
@@ -3019,7 +3331,7 @@
         </is>
       </c>
       <c r="C2" s="3" t="n">
-        <v>1</v>
+        <v>0.9608018940605703</v>
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
@@ -3047,7 +3359,7 @@
         </is>
       </c>
       <c r="C3" s="3" t="n">
-        <v>0.08344982949310291</v>
+        <v>0.04784722458896093</v>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
@@ -3055,7 +3367,7 @@
         </is>
       </c>
       <c r="E3" s="3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
@@ -3075,7 +3387,7 @@
         </is>
       </c>
       <c r="C4" s="3" t="n">
-        <v>0.9484912846303624</v>
+        <v>0.6263814204856222</v>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
@@ -3103,7 +3415,7 @@
         </is>
       </c>
       <c r="C5" s="3" t="n">
-        <v>0.01203866536063322</v>
+        <v>0.00488110702362953</v>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
@@ -3131,7 +3443,7 @@
         </is>
       </c>
       <c r="C6" s="3" t="n">
-        <v>0.02373635160823725</v>
+        <v>0.02938892047286141</v>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
@@ -3159,7 +3471,7 @@
         </is>
       </c>
       <c r="C7" s="3" t="n">
-        <v>0.7464142297508616</v>
+        <v>0.4572444216238805</v>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
@@ -3187,7 +3499,7 @@
         </is>
       </c>
       <c r="C8" s="3" t="n">
-        <v>0.01409405340133985</v>
+        <v>0.006809150097497262</v>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
@@ -3215,7 +3527,7 @@
         </is>
       </c>
       <c r="C9" s="3" t="n">
-        <v>0.4275564756355391</v>
+        <v>0.558947374068095</v>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
@@ -3243,7 +3555,7 @@
         </is>
       </c>
       <c r="C10" s="3" t="n">
-        <v>0.0047312126626677</v>
+        <v>0.002827330717951227</v>
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
@@ -3271,7 +3583,7 @@
         </is>
       </c>
       <c r="C11" s="3" t="n">
-        <v>0.009764472414768617</v>
+        <v>0.003544521685164924</v>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
@@ -3299,7 +3611,7 @@
         </is>
       </c>
       <c r="C12" s="3" t="n">
-        <v>0.09302753827955859</v>
+        <v>0.05651855511195005</v>
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
@@ -3327,7 +3639,7 @@
         </is>
       </c>
       <c r="C13" s="3" t="n">
-        <v>0.4294884617174285</v>
+        <v>0.2873273855988826</v>
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
@@ -3355,7 +3667,7 @@
         </is>
       </c>
       <c r="C14" s="3" t="n">
-        <v>0.5609617572539256</v>
+        <v>0.4936154695260365</v>
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
@@ -3383,7 +3695,7 @@
         </is>
       </c>
       <c r="C15" s="3" t="n">
-        <v>0.005161410370458398</v>
+        <v>0.001522588585183457</v>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
@@ -3411,7 +3723,7 @@
         </is>
       </c>
       <c r="C16" s="3" t="n">
-        <v>0.5617369040242319</v>
+        <v>0.7256159408473616</v>
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
@@ -3439,7 +3751,7 @@
         </is>
       </c>
       <c r="C17" s="3" t="n">
-        <v>0.2704850051020423</v>
+        <v>0.2622863556732082</v>
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
@@ -3467,7 +3779,7 @@
         </is>
       </c>
       <c r="C18" s="3" t="n">
-        <v>0.7933505521096174</v>
+        <v>0.5208480313753976</v>
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
@@ -3495,7 +3807,7 @@
         </is>
       </c>
       <c r="C19" s="3" t="n">
-        <v>0.5138874845508352</v>
+        <v>0.3200302155933907</v>
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
@@ -3523,7 +3835,7 @@
         </is>
       </c>
       <c r="C20" s="3" t="n">
-        <v>0.08172028164814853</v>
+        <v>0.1985503644638253</v>
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
@@ -3551,7 +3863,7 @@
         </is>
       </c>
       <c r="C21" s="3" t="n">
-        <v>0.009277402490967462</v>
+        <v>0.00402709286994327</v>
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
@@ -3585,7 +3897,7 @@
     <col width="23" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="23" customWidth="1" min="5" max="5"/>
     <col width="25" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -3638,13 +3950,13 @@
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>2.688146786492376</v>
+        <v>3.95670387914768</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>0.05083006516901065</v>
+        <v>0.009420541846232398</v>
       </c>
       <c r="F2" s="3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3">
@@ -3664,10 +3976,10 @@
         </is>
       </c>
       <c r="D3" s="3" t="n">
-        <v>1.734757768579079</v>
+        <v>2.257194392720053</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>0.169355720984522</v>
+        <v>0.08269593347326513</v>
       </c>
       <c r="F3" s="3" t="b">
         <v>0</v>
@@ -3690,13 +4002,13 @@
         </is>
       </c>
       <c r="D4" s="3" t="n">
-        <v>1.798764620092082</v>
+        <v>2.708393082524991</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>0.1561189987849128</v>
+        <v>0.04582870018036539</v>
       </c>
       <c r="F4" s="3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5">
@@ -3716,10 +4028,10 @@
         </is>
       </c>
       <c r="D5" s="3" t="n">
-        <v>2.848244131094633</v>
+        <v>3.178952996463713</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>0.04169025680677561</v>
+        <v>0.02498570255569007</v>
       </c>
       <c r="F5" s="3" t="b">
         <v>1</v>
@@ -3742,10 +4054,10 @@
         </is>
       </c>
       <c r="D6" s="3" t="n">
-        <v>2.606643746611922</v>
+        <v>1.878348101265823</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>0.05625883226422726</v>
+        <v>0.1361469280875903</v>
       </c>
       <c r="F6" s="3" t="b">
         <v>0</v>
@@ -3768,10 +4080,10 @@
         </is>
       </c>
       <c r="D7" s="3" t="n">
-        <v>1.149964085067084</v>
+        <v>1.339111507726844</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>0.3530467701759638</v>
+        <v>0.2749236113576879</v>
       </c>
       <c r="F7" s="3" t="b">
         <v>0</v>
@@ -3794,13 +4106,13 @@
         </is>
       </c>
       <c r="D8" s="3" t="n">
-        <v>2.560823110189312</v>
+        <v>3.11234964218647</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>0.05957105547785645</v>
+        <v>0.02720711948876369</v>
       </c>
       <c r="F8" s="3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9">
@@ -3820,10 +4132,10 @@
         </is>
       </c>
       <c r="D9" s="3" t="n">
-        <v>3.368164121905224</v>
+        <v>4.020055095788944</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>0.02214800086622022</v>
+        <v>0.008715363880588878</v>
       </c>
       <c r="F9" s="3" t="b">
         <v>1</v>
@@ -3854,10 +4166,10 @@
         </is>
       </c>
       <c r="D11" s="3" t="n">
-        <v>-0.8323148993037752</v>
+        <v>-1.091089451179962</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>0.4370983363053137</v>
+        <v>0.3070016039744494</v>
       </c>
       <c r="F11" s="3" t="b">
         <v>0</v>
@@ -3880,10 +4192,10 @@
         </is>
       </c>
       <c r="D12" s="3" t="n">
-        <v>-0.8293962196513643</v>
+        <v>-0.3713906763541034</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>0.438624415622445</v>
+        <v>0.7199897873752998</v>
       </c>
       <c r="F12" s="3" t="b">
         <v>0</v>
@@ -3906,10 +4218,10 @@
         </is>
       </c>
       <c r="D13" s="3" t="n">
-        <v>0.6333004963811245</v>
+        <v>0.240336707250445</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>0.549899173505021</v>
+        <v>0.8161134404714866</v>
       </c>
       <c r="F13" s="3" t="b">
         <v>0</v>
@@ -3932,10 +4244,10 @@
         </is>
       </c>
       <c r="D14" s="3" t="n">
-        <v>0.1786474002526238</v>
+        <v>0</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>0.8640941349883791</v>
+        <v>1</v>
       </c>
       <c r="F14" s="3" t="b">
         <v>0</v>
@@ -3966,10 +4278,10 @@
         </is>
       </c>
       <c r="D16" s="3" t="n">
-        <v>0.8103965430069947</v>
+        <v>1.344361034193523</v>
       </c>
       <c r="E16" s="3" t="n">
-        <v>0.4545388771419559</v>
+        <v>0.2274282079155049</v>
       </c>
       <c r="F16" s="3" t="b">
         <v>0</v>
@@ -3992,10 +4304,10 @@
         </is>
       </c>
       <c r="D17" s="3" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>0.8125</v>
+        <v>0.84375</v>
       </c>
       <c r="F17" s="3" t="b">
         <v>0</v>
@@ -4018,10 +4330,10 @@
         </is>
       </c>
       <c r="D18" s="3" t="n">
-        <v>0.817623560871883</v>
+        <v>1.222631418787729</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>0.4507615688534394</v>
+        <v>0.2673114535246533</v>
       </c>
       <c r="F18" s="3" t="b">
         <v>0</v>
@@ -4040,14 +4352,14 @@
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>Wilcoxon</t>
+          <t>T-test</t>
         </is>
       </c>
       <c r="D19" s="3" t="n">
-        <v>1.5</v>
+        <v>1.757315203104789</v>
       </c>
       <c r="E19" s="3" t="n">
-        <v>0.375</v>
+        <v>0.1293748508953314</v>
       </c>
       <c r="F19" s="3" t="b">
         <v>0</v>
@@ -4078,10 +4390,10 @@
         </is>
       </c>
       <c r="D21" s="3" t="n">
-        <v>0.8798826901281195</v>
+        <v>1.197148331910294</v>
       </c>
       <c r="E21" s="3" t="n">
-        <v>0.412773025377815</v>
+        <v>0.270212591389518</v>
       </c>
       <c r="F21" s="3" t="b">
         <v>0</v>
@@ -4104,10 +4416,10 @@
         </is>
       </c>
       <c r="D22" s="3" t="n">
-        <v>-0.547722557505167</v>
+        <v>0.4349588362008398</v>
       </c>
       <c r="E22" s="3" t="n">
-        <v>0.6036450565101357</v>
+        <v>0.676686935028977</v>
       </c>
       <c r="F22" s="3" t="b">
         <v>0</v>
@@ -4130,10 +4442,10 @@
         </is>
       </c>
       <c r="D23" s="3" t="n">
-        <v>-0.7604691006293732</v>
+        <v>-0.7637626158259733</v>
       </c>
       <c r="E23" s="3" t="n">
-        <v>0.4757860843342303</v>
+        <v>0.4699636420584196</v>
       </c>
       <c r="F23" s="3" t="b">
         <v>0</v>
@@ -4156,13 +4468,13 @@
         </is>
       </c>
       <c r="D24" s="3" t="n">
-        <v>3.286335345030996</v>
+        <v>1.9296124624699</v>
       </c>
       <c r="E24" s="3" t="n">
-        <v>0.01668998431583146</v>
+        <v>0.094976492435775</v>
       </c>
       <c r="F24" s="3" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25">
@@ -4190,10 +4502,10 @@
         </is>
       </c>
       <c r="D26" s="3" t="n">
-        <v>1.23582876130665</v>
+        <v>1.229232775294831</v>
       </c>
       <c r="E26" s="3" t="n">
-        <v>0.2627088836889246</v>
+        <v>0.2586973904995958</v>
       </c>
       <c r="F26" s="3" t="b">
         <v>0</v>
@@ -4216,10 +4528,10 @@
         </is>
       </c>
       <c r="D27" s="3" t="n">
-        <v>6.18146635643918</v>
+        <v>3.517568943509836</v>
       </c>
       <c r="E27" s="3" t="n">
-        <v>0.0008244673687807453</v>
+        <v>0.009759500959109107</v>
       </c>
       <c r="F27" s="3" t="b">
         <v>1</v>
@@ -4242,10 +4554,10 @@
         </is>
       </c>
       <c r="D28" s="3" t="n">
-        <v>3.103187231277934</v>
+        <v>2.861426353911546</v>
       </c>
       <c r="E28" s="3" t="n">
-        <v>0.02103077046268435</v>
+        <v>0.02428798676342096</v>
       </c>
       <c r="F28" s="3" t="b">
         <v>1</v>
@@ -4268,10 +4580,10 @@
         </is>
       </c>
       <c r="D29" s="3" t="n">
-        <v>3.945575695328575</v>
+        <v>4.630064794363034</v>
       </c>
       <c r="E29" s="3" t="n">
-        <v>0.007575990448404784</v>
+        <v>0.002397503591143557</v>
       </c>
       <c r="F29" s="3" t="b">
         <v>1</v>
@@ -4302,10 +4614,10 @@
         </is>
       </c>
       <c r="D31" s="3" t="n">
-        <v>-0.1206776980063695</v>
+        <v>0.1179682202715451</v>
       </c>
       <c r="E31" s="3" t="n">
-        <v>0.9078861043896856</v>
+        <v>0.9094065494908765</v>
       </c>
       <c r="F31" s="3" t="b">
         <v>0</v>
@@ -4324,14 +4636,14 @@
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>T-test</t>
+          <t>Wilcoxon</t>
         </is>
       </c>
       <c r="D32" s="3" t="n">
-        <v>1.071884401515744</v>
+        <v>8.5</v>
       </c>
       <c r="E32" s="3" t="n">
-        <v>0.3249810681138469</v>
+        <v>0.203125</v>
       </c>
       <c r="F32" s="3" t="b">
         <v>0</v>
@@ -4354,10 +4666,10 @@
         </is>
       </c>
       <c r="D33" s="3" t="n">
-        <v>-0.7965329572329224</v>
+        <v>-0.7008766440504623</v>
       </c>
       <c r="E33" s="3" t="n">
-        <v>0.4560744262302296</v>
+        <v>0.5060027660022388</v>
       </c>
       <c r="F33" s="3" t="b">
         <v>0</v>
@@ -4380,10 +4692,10 @@
         </is>
       </c>
       <c r="D34" s="3" t="n">
-        <v>1.306549159836976</v>
+        <v>1.297223207936515</v>
       </c>
       <c r="E34" s="3" t="n">
-        <v>0.2392100249855083</v>
+        <v>0.2356695290289083</v>
       </c>
       <c r="F34" s="3" t="b">
         <v>0</v>

</xml_diff>

<commit_message>
New partecipants; results updated
</commit_message>
<xml_diff>
--- a/app/analysis/Questionnaire_results.xlsx
+++ b/app/analysis/Questionnaire_results.xlsx
@@ -434,7 +434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P41"/>
+  <dimension ref="A1:P46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1007,59 +1007,59 @@
     </row>
     <row r="11">
       <c r="A11" s="3" t="n">
-        <v>7</v>
+        <v>46</v>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>CS0</t>
+          <t>CC</t>
         </is>
       </c>
       <c r="C11" s="3" t="n">
         <v>3.25</v>
       </c>
       <c r="D11" s="3" t="n">
-        <v>3.25</v>
+        <v>3.5</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>3.5</v>
+        <v>4.5</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>1.75</v>
+        <v>4.5</v>
       </c>
       <c r="G11" s="3" t="n">
+        <v>4.25</v>
+      </c>
+      <c r="H11" s="3" t="n">
         <v>4</v>
-      </c>
-      <c r="H11" s="3" t="n">
-        <v>1</v>
       </c>
       <c r="I11" s="3" t="n">
         <v>3.4</v>
       </c>
       <c r="J11" s="3" t="n">
-        <v>3</v>
+        <v>3.6</v>
       </c>
       <c r="K11" s="3" t="n">
-        <v>3</v>
+        <v>3.8</v>
       </c>
       <c r="L11" s="3" t="n">
-        <v>3</v>
+        <v>3.6</v>
       </c>
       <c r="M11" s="3" t="n">
-        <v>3</v>
+        <v>3.8</v>
       </c>
       <c r="N11" s="3" t="n">
-        <v>3.4</v>
+        <v>4</v>
       </c>
       <c r="O11" s="3" t="n">
-        <v>2.8</v>
+        <v>2</v>
       </c>
       <c r="P11" s="3" t="n">
-        <v>1.6</v>
+        <v>3.6</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="n">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
@@ -1067,51 +1067,51 @@
         </is>
       </c>
       <c r="C12" s="3" t="n">
-        <v>2.5</v>
+        <v>3.25</v>
       </c>
       <c r="D12" s="3" t="n">
-        <v>2</v>
+        <v>3.25</v>
       </c>
       <c r="E12" s="3" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="F12" s="3" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="G12" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="F12" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="G12" s="3" t="n">
-        <v>4.25</v>
-      </c>
       <c r="H12" s="3" t="n">
-        <v>4.5</v>
+        <v>1</v>
       </c>
       <c r="I12" s="3" t="n">
-        <v>4.6</v>
+        <v>3.4</v>
       </c>
       <c r="J12" s="3" t="n">
-        <v>4.8</v>
+        <v>3</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>4.4</v>
+        <v>3</v>
       </c>
       <c r="L12" s="3" t="n">
-        <v>4.8</v>
+        <v>3</v>
       </c>
       <c r="M12" s="3" t="n">
-        <v>3.2</v>
+        <v>3</v>
       </c>
       <c r="N12" s="3" t="n">
-        <v>3.2</v>
+        <v>3.4</v>
       </c>
       <c r="O12" s="3" t="n">
-        <v>4.2</v>
+        <v>2.8</v>
       </c>
       <c r="P12" s="3" t="n">
-        <v>4.2</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="n">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
@@ -1119,51 +1119,51 @@
         </is>
       </c>
       <c r="C13" s="3" t="n">
-        <v>2</v>
+        <v>2.5</v>
       </c>
       <c r="D13" s="3" t="n">
         <v>2</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>2.25</v>
+        <v>4</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>3.5</v>
+        <v>4.25</v>
       </c>
       <c r="H13" s="3" t="n">
-        <v>3.75</v>
+        <v>4.5</v>
       </c>
       <c r="I13" s="3" t="n">
-        <v>3</v>
+        <v>4.6</v>
       </c>
       <c r="J13" s="3" t="n">
-        <v>3</v>
+        <v>4.8</v>
       </c>
       <c r="K13" s="3" t="n">
-        <v>3.8</v>
+        <v>4.4</v>
       </c>
       <c r="L13" s="3" t="n">
-        <v>3.6</v>
+        <v>4.8</v>
       </c>
       <c r="M13" s="3" t="n">
-        <v>3.4</v>
+        <v>3.2</v>
       </c>
       <c r="N13" s="3" t="n">
-        <v>4</v>
+        <v>3.2</v>
       </c>
       <c r="O13" s="3" t="n">
-        <v>3</v>
+        <v>4.2</v>
       </c>
       <c r="P13" s="3" t="n">
-        <v>3.4</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="n">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
@@ -1171,13 +1171,13 @@
         </is>
       </c>
       <c r="C14" s="3" t="n">
-        <v>2.5</v>
+        <v>2</v>
       </c>
       <c r="D14" s="3" t="n">
-        <v>2.5</v>
+        <v>2</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>3.25</v>
+        <v>2.25</v>
       </c>
       <c r="F14" s="3" t="n">
         <v>3</v>
@@ -1186,36 +1186,36 @@
         <v>3.5</v>
       </c>
       <c r="H14" s="3" t="n">
-        <v>2.5</v>
+        <v>3.75</v>
       </c>
       <c r="I14" s="3" t="n">
-        <v>3.4</v>
+        <v>3</v>
       </c>
       <c r="J14" s="3" t="n">
         <v>3</v>
       </c>
       <c r="K14" s="3" t="n">
-        <v>3.2</v>
+        <v>3.8</v>
       </c>
       <c r="L14" s="3" t="n">
         <v>3.6</v>
       </c>
       <c r="M14" s="3" t="n">
-        <v>3.8</v>
+        <v>3.4</v>
       </c>
       <c r="N14" s="3" t="n">
         <v>4</v>
       </c>
       <c r="O14" s="3" t="n">
-        <v>3.6</v>
+        <v>3</v>
       </c>
       <c r="P14" s="3" t="n">
-        <v>3.2</v>
+        <v>3.4</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="n">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
@@ -1223,51 +1223,51 @@
         </is>
       </c>
       <c r="C15" s="3" t="n">
-        <v>3</v>
+        <v>2.5</v>
       </c>
       <c r="D15" s="3" t="n">
-        <v>3</v>
+        <v>2.5</v>
       </c>
       <c r="E15" s="3" t="n">
-        <v>4</v>
+        <v>3.25</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>4</v>
+        <v>3.5</v>
       </c>
       <c r="H15" s="3" t="n">
-        <v>4</v>
+        <v>2.5</v>
       </c>
       <c r="I15" s="3" t="n">
         <v>3.4</v>
       </c>
       <c r="J15" s="3" t="n">
-        <v>4.4</v>
+        <v>3</v>
       </c>
       <c r="K15" s="3" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="L15" s="3" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="M15" s="3" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="N15" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="L15" s="3" t="n">
-        <v>4.4</v>
-      </c>
-      <c r="M15" s="3" t="n">
-        <v>4.4</v>
-      </c>
-      <c r="N15" s="3" t="n">
+      <c r="O15" s="3" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="P15" s="3" t="n">
         <v>3.2</v>
-      </c>
-      <c r="O15" s="3" t="n">
-        <v>3.4</v>
-      </c>
-      <c r="P15" s="3" t="n">
-        <v>3.4</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="n">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
@@ -1275,51 +1275,51 @@
         </is>
       </c>
       <c r="C16" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="D16" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E16" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="D16" s="3" t="n">
-        <v>4.25</v>
-      </c>
-      <c r="E16" s="3" t="n">
-        <v>5</v>
-      </c>
       <c r="F16" s="3" t="n">
-        <v>2.5</v>
+        <v>4</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H16" s="3" t="n">
-        <v>2.25</v>
+        <v>4</v>
       </c>
       <c r="I16" s="3" t="n">
-        <v>5</v>
+        <v>3.4</v>
       </c>
       <c r="J16" s="3" t="n">
-        <v>1.6</v>
+        <v>4.4</v>
       </c>
       <c r="K16" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="L16" s="3" t="n">
         <v>4.4</v>
       </c>
-      <c r="L16" s="3" t="n">
-        <v>1.6</v>
-      </c>
       <c r="M16" s="3" t="n">
-        <v>4.8</v>
+        <v>4.4</v>
       </c>
       <c r="N16" s="3" t="n">
-        <v>2.6</v>
+        <v>3.2</v>
       </c>
       <c r="O16" s="3" t="n">
-        <v>5</v>
+        <v>3.4</v>
       </c>
       <c r="P16" s="3" t="n">
-        <v>1.2</v>
+        <v>3.4</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="n">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
@@ -1327,155 +1327,155 @@
         </is>
       </c>
       <c r="C17" s="3" t="n">
-        <v>2.75</v>
+        <v>4</v>
       </c>
       <c r="D17" s="3" t="n">
-        <v>2.75</v>
+        <v>4.25</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>1.5</v>
+        <v>2.5</v>
       </c>
       <c r="G17" s="3" t="n">
-        <v>3.25</v>
+        <v>5</v>
       </c>
       <c r="H17" s="3" t="n">
-        <v>1.25</v>
+        <v>2.25</v>
       </c>
       <c r="I17" s="3" t="n">
-        <v>4.6</v>
+        <v>5</v>
       </c>
       <c r="J17" s="3" t="n">
-        <v>1.8</v>
+        <v>1.6</v>
       </c>
       <c r="K17" s="3" t="n">
         <v>4.4</v>
       </c>
       <c r="L17" s="3" t="n">
-        <v>2.2</v>
+        <v>1.6</v>
       </c>
       <c r="M17" s="3" t="n">
-        <v>2.8</v>
+        <v>4.8</v>
       </c>
       <c r="N17" s="3" t="n">
-        <v>1.6</v>
+        <v>2.6</v>
       </c>
       <c r="O17" s="3" t="n">
-        <v>2.8</v>
+        <v>5</v>
       </c>
       <c r="P17" s="3" t="n">
-        <v>1</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="n">
-        <v>3</v>
+        <v>37</v>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>CS1</t>
+          <t>CS0</t>
         </is>
       </c>
       <c r="C18" s="3" t="n">
-        <v>3.5</v>
+        <v>2.75</v>
       </c>
       <c r="D18" s="3" t="n">
-        <v>3</v>
+        <v>2.75</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>4.5</v>
+        <v>3</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>3</v>
+        <v>1.5</v>
       </c>
       <c r="G18" s="3" t="n">
         <v>3.25</v>
       </c>
       <c r="H18" s="3" t="n">
-        <v>3</v>
+        <v>1.25</v>
       </c>
       <c r="I18" s="3" t="n">
-        <v>4</v>
+        <v>4.6</v>
       </c>
       <c r="J18" s="3" t="n">
-        <v>2.4</v>
+        <v>1.8</v>
       </c>
       <c r="K18" s="3" t="n">
-        <v>3.6</v>
+        <v>4.4</v>
       </c>
       <c r="L18" s="3" t="n">
-        <v>3.6</v>
+        <v>2.2</v>
       </c>
       <c r="M18" s="3" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="N18" s="3" t="n">
         <v>1.6</v>
       </c>
-      <c r="N18" s="3" t="n">
-        <v>2</v>
-      </c>
       <c r="O18" s="3" t="n">
-        <v>4</v>
+        <v>2.8</v>
       </c>
       <c r="P18" s="3" t="n">
-        <v>3.8</v>
+        <v>1</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="n">
-        <v>8</v>
+        <v>42</v>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>CS1</t>
+          <t>CS0</t>
         </is>
       </c>
       <c r="C19" s="3" t="n">
-        <v>3.25</v>
+        <v>3.75</v>
       </c>
       <c r="D19" s="3" t="n">
-        <v>2.5</v>
+        <v>1.25</v>
       </c>
       <c r="E19" s="3" t="n">
-        <v>2.75</v>
+        <v>3</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>2.75</v>
+        <v>1</v>
       </c>
       <c r="G19" s="3" t="n">
-        <v>3</v>
+        <v>3.75</v>
       </c>
       <c r="H19" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I19" s="3" t="n">
-        <v>1.6</v>
+        <v>2.2</v>
       </c>
       <c r="J19" s="3" t="n">
-        <v>1.6</v>
+        <v>2.8</v>
       </c>
       <c r="K19" s="3" t="n">
-        <v>1.8</v>
+        <v>3.6</v>
       </c>
       <c r="L19" s="3" t="n">
-        <v>2</v>
+        <v>2.2</v>
       </c>
       <c r="M19" s="3" t="n">
         <v>2.6</v>
       </c>
       <c r="N19" s="3" t="n">
-        <v>2.4</v>
+        <v>1.8</v>
       </c>
       <c r="O19" s="3" t="n">
-        <v>2.8</v>
+        <v>3</v>
       </c>
       <c r="P19" s="3" t="n">
-        <v>2.6</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="n">
-        <v>13</v>
+        <v>3</v>
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
@@ -1483,51 +1483,51 @@
         </is>
       </c>
       <c r="C20" s="3" t="n">
-        <v>2.75</v>
+        <v>3.5</v>
       </c>
       <c r="D20" s="3" t="n">
         <v>3</v>
       </c>
       <c r="E20" s="3" t="n">
-        <v>2.5</v>
+        <v>4.5</v>
       </c>
       <c r="F20" s="3" t="n">
-        <v>3.5</v>
+        <v>3</v>
       </c>
       <c r="G20" s="3" t="n">
-        <v>2.75</v>
+        <v>3.25</v>
       </c>
       <c r="H20" s="3" t="n">
-        <v>2.75</v>
+        <v>3</v>
       </c>
       <c r="I20" s="3" t="n">
-        <v>3.2</v>
+        <v>4</v>
       </c>
       <c r="J20" s="3" t="n">
-        <v>3.4</v>
+        <v>2.4</v>
       </c>
       <c r="K20" s="3" t="n">
-        <v>2.6</v>
+        <v>3.6</v>
       </c>
       <c r="L20" s="3" t="n">
-        <v>3.4</v>
+        <v>3.6</v>
       </c>
       <c r="M20" s="3" t="n">
-        <v>2.4</v>
+        <v>1.6</v>
       </c>
       <c r="N20" s="3" t="n">
-        <v>3.2</v>
+        <v>2</v>
       </c>
       <c r="O20" s="3" t="n">
-        <v>3.4</v>
+        <v>4</v>
       </c>
       <c r="P20" s="3" t="n">
-        <v>3.4</v>
+        <v>3.8</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="n">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
@@ -1535,51 +1535,51 @@
         </is>
       </c>
       <c r="C21" s="3" t="n">
-        <v>1</v>
+        <v>3.25</v>
       </c>
       <c r="D21" s="3" t="n">
-        <v>1</v>
+        <v>2.5</v>
       </c>
       <c r="E21" s="3" t="n">
-        <v>4</v>
+        <v>2.75</v>
       </c>
       <c r="F21" s="3" t="n">
-        <v>3</v>
+        <v>2.75</v>
       </c>
       <c r="G21" s="3" t="n">
-        <v>2.75</v>
+        <v>3</v>
       </c>
       <c r="H21" s="3" t="n">
-        <v>2.5</v>
+        <v>2</v>
       </c>
       <c r="I21" s="3" t="n">
-        <v>2.4</v>
+        <v>1.6</v>
       </c>
       <c r="J21" s="3" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="K21" s="3" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="L21" s="3" t="n">
         <v>2</v>
-      </c>
-      <c r="K21" s="3" t="n">
-        <v>2.6</v>
-      </c>
-      <c r="L21" s="3" t="n">
-        <v>2.2</v>
       </c>
       <c r="M21" s="3" t="n">
         <v>2.6</v>
       </c>
       <c r="N21" s="3" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="O21" s="3" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="P21" s="3" t="n">
         <v>2.6</v>
-      </c>
-      <c r="O21" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="P21" s="3" t="n">
-        <v>2.8</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="n">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
@@ -1587,51 +1587,51 @@
         </is>
       </c>
       <c r="C22" s="3" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="D22" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E22" s="3" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F22" s="3" t="n">
         <v>3.5</v>
       </c>
-      <c r="D22" s="3" t="n">
-        <v>3.75</v>
-      </c>
-      <c r="E22" s="3" t="n">
-        <v>4.75</v>
-      </c>
-      <c r="F22" s="3" t="n">
-        <v>4.75</v>
-      </c>
       <c r="G22" s="3" t="n">
-        <v>4.5</v>
+        <v>2.75</v>
       </c>
       <c r="H22" s="3" t="n">
-        <v>4.5</v>
+        <v>2.75</v>
       </c>
       <c r="I22" s="3" t="n">
         <v>3.2</v>
       </c>
       <c r="J22" s="3" t="n">
-        <v>3</v>
+        <v>3.4</v>
       </c>
       <c r="K22" s="3" t="n">
-        <v>3</v>
+        <v>2.6</v>
       </c>
       <c r="L22" s="3" t="n">
-        <v>2.8</v>
+        <v>3.4</v>
       </c>
       <c r="M22" s="3" t="n">
-        <v>4</v>
+        <v>2.4</v>
       </c>
       <c r="N22" s="3" t="n">
-        <v>4</v>
+        <v>3.2</v>
       </c>
       <c r="O22" s="3" t="n">
-        <v>3</v>
+        <v>3.4</v>
       </c>
       <c r="P22" s="3" t="n">
-        <v>3</v>
+        <v>3.4</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="n">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
@@ -1639,51 +1639,51 @@
         </is>
       </c>
       <c r="C23" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D23" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E23" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="F23" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="G23" s="3" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="H23" s="3" t="n">
         <v>2.5</v>
       </c>
-      <c r="D23" s="3" t="n">
-        <v>1.75</v>
-      </c>
-      <c r="E23" s="3" t="n">
-        <v>4.75</v>
-      </c>
-      <c r="F23" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="G23" s="3" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="H23" s="3" t="n">
-        <v>4.5</v>
-      </c>
       <c r="I23" s="3" t="n">
-        <v>3</v>
+        <v>2.4</v>
       </c>
       <c r="J23" s="3" t="n">
-        <v>3.6</v>
+        <v>2</v>
       </c>
       <c r="K23" s="3" t="n">
-        <v>3.8</v>
+        <v>2.6</v>
       </c>
       <c r="L23" s="3" t="n">
-        <v>4.2</v>
+        <v>2.2</v>
       </c>
       <c r="M23" s="3" t="n">
-        <v>2.2</v>
+        <v>2.6</v>
       </c>
       <c r="N23" s="3" t="n">
-        <v>1.8</v>
+        <v>2.6</v>
       </c>
       <c r="O23" s="3" t="n">
-        <v>3.8</v>
+        <v>3</v>
       </c>
       <c r="P23" s="3" t="n">
-        <v>3.6</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="n">
-        <v>33</v>
+        <v>23</v>
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
@@ -1691,16 +1691,16 @@
         </is>
       </c>
       <c r="C24" s="3" t="n">
-        <v>4</v>
+        <v>3.5</v>
       </c>
       <c r="D24" s="3" t="n">
         <v>3.75</v>
       </c>
       <c r="E24" s="3" t="n">
-        <v>5</v>
+        <v>4.75</v>
       </c>
       <c r="F24" s="3" t="n">
-        <v>5</v>
+        <v>4.75</v>
       </c>
       <c r="G24" s="3" t="n">
         <v>4.5</v>
@@ -1709,33 +1709,33 @@
         <v>4.5</v>
       </c>
       <c r="I24" s="3" t="n">
-        <v>4.6</v>
+        <v>3.2</v>
       </c>
       <c r="J24" s="3" t="n">
-        <v>4.4</v>
+        <v>3</v>
       </c>
       <c r="K24" s="3" t="n">
-        <v>4.6</v>
+        <v>3</v>
       </c>
       <c r="L24" s="3" t="n">
-        <v>4.4</v>
+        <v>2.8</v>
       </c>
       <c r="M24" s="3" t="n">
-        <v>3.8</v>
+        <v>4</v>
       </c>
       <c r="N24" s="3" t="n">
         <v>4</v>
       </c>
       <c r="O24" s="3" t="n">
-        <v>2.8</v>
+        <v>3</v>
       </c>
       <c r="P24" s="3" t="n">
-        <v>2.4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="n">
-        <v>38</v>
+        <v>28</v>
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
@@ -1743,207 +1743,207 @@
         </is>
       </c>
       <c r="C25" s="3" t="n">
-        <v>2.25</v>
+        <v>2.5</v>
       </c>
       <c r="D25" s="3" t="n">
-        <v>2.5</v>
+        <v>1.75</v>
       </c>
       <c r="E25" s="3" t="n">
-        <v>3.75</v>
+        <v>4.75</v>
       </c>
       <c r="F25" s="3" t="n">
-        <v>3.75</v>
+        <v>4</v>
       </c>
       <c r="G25" s="3" t="n">
-        <v>4</v>
+        <v>4.5</v>
       </c>
       <c r="H25" s="3" t="n">
-        <v>3</v>
+        <v>4.5</v>
       </c>
       <c r="I25" s="3" t="n">
-        <v>3.2</v>
+        <v>3</v>
       </c>
       <c r="J25" s="3" t="n">
-        <v>2.6</v>
+        <v>3.6</v>
       </c>
       <c r="K25" s="3" t="n">
-        <v>4.4</v>
+        <v>3.8</v>
       </c>
       <c r="L25" s="3" t="n">
-        <v>3</v>
+        <v>4.2</v>
       </c>
       <c r="M25" s="3" t="n">
-        <v>2.8</v>
+        <v>2.2</v>
       </c>
       <c r="N25" s="3" t="n">
-        <v>2.8</v>
+        <v>1.8</v>
       </c>
       <c r="O25" s="3" t="n">
-        <v>3.2</v>
+        <v>3.8</v>
       </c>
       <c r="P25" s="3" t="n">
-        <v>3.4</v>
+        <v>3.6</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="n">
+        <v>33</v>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>CS1</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="B26" s="3" t="inlineStr">
-        <is>
-          <t>CI</t>
-        </is>
-      </c>
-      <c r="C26" s="3" t="n">
-        <v>2.75</v>
-      </c>
       <c r="D26" s="3" t="n">
-        <v>2</v>
+        <v>3.75</v>
       </c>
       <c r="E26" s="3" t="n">
-        <v>3.75</v>
+        <v>5</v>
       </c>
       <c r="F26" s="3" t="n">
-        <v>3.5</v>
+        <v>5</v>
       </c>
       <c r="G26" s="3" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="H26" s="3" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="I26" s="3" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="J26" s="3" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="K26" s="3" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="L26" s="3" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="M26" s="3" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="N26" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="H26" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="I26" s="3" t="n">
-        <v>4.4</v>
-      </c>
-      <c r="J26" s="3" t="n">
-        <v>3.2</v>
-      </c>
-      <c r="K26" s="3" t="n">
-        <v>4.2</v>
-      </c>
-      <c r="L26" s="3" t="n">
+      <c r="O26" s="3" t="n">
         <v>2.8</v>
       </c>
-      <c r="M26" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="N26" s="3" t="n">
-        <v>2.2</v>
-      </c>
-      <c r="O26" s="3" t="n">
-        <v>4</v>
-      </c>
       <c r="P26" s="3" t="n">
-        <v>3.6</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="n">
-        <v>9</v>
+        <v>38</v>
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>CI</t>
+          <t>CS1</t>
         </is>
       </c>
       <c r="C27" s="3" t="n">
-        <v>2.5</v>
+        <v>2.25</v>
       </c>
       <c r="D27" s="3" t="n">
         <v>2.5</v>
       </c>
       <c r="E27" s="3" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="F27" s="3" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="G27" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="F27" s="3" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="G27" s="3" t="n">
-        <v>3.5</v>
-      </c>
       <c r="H27" s="3" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I27" s="3" t="n">
-        <v>2.2</v>
+        <v>3.2</v>
       </c>
       <c r="J27" s="3" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="K27" s="3" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="L27" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="M27" s="3" t="n">
         <v>2.8</v>
       </c>
-      <c r="K27" s="3" t="n">
+      <c r="N27" s="3" t="n">
         <v>2.8</v>
       </c>
-      <c r="L27" s="3" t="n">
-        <v>2.4</v>
-      </c>
-      <c r="M27" s="3" t="n">
+      <c r="O27" s="3" t="n">
         <v>3.2</v>
       </c>
-      <c r="N27" s="3" t="n">
-        <v>1.8</v>
-      </c>
-      <c r="O27" s="3" t="n">
+      <c r="P27" s="3" t="n">
         <v>3.4</v>
-      </c>
-      <c r="P27" s="3" t="n">
-        <v>2.4</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="3" t="n">
-        <v>14</v>
+        <v>43</v>
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>CI</t>
+          <t>CS1</t>
         </is>
       </c>
       <c r="C28" s="3" t="n">
         <v>3</v>
       </c>
       <c r="D28" s="3" t="n">
-        <v>3.25</v>
+        <v>2.25</v>
       </c>
       <c r="E28" s="3" t="n">
         <v>3.5</v>
       </c>
       <c r="F28" s="3" t="n">
-        <v>3</v>
+        <v>2.5</v>
       </c>
       <c r="G28" s="3" t="n">
-        <v>3.25</v>
+        <v>3</v>
       </c>
       <c r="H28" s="3" t="n">
-        <v>3</v>
+        <v>2.5</v>
       </c>
       <c r="I28" s="3" t="n">
-        <v>3.4</v>
+        <v>2.6</v>
       </c>
       <c r="J28" s="3" t="n">
-        <v>2.2</v>
+        <v>2</v>
       </c>
       <c r="K28" s="3" t="n">
-        <v>3.6</v>
+        <v>3.2</v>
       </c>
       <c r="L28" s="3" t="n">
         <v>2</v>
       </c>
       <c r="M28" s="3" t="n">
-        <v>3.8</v>
+        <v>2.2</v>
       </c>
       <c r="N28" s="3" t="n">
-        <v>2.8</v>
+        <v>1.4</v>
       </c>
       <c r="O28" s="3" t="n">
-        <v>2.8</v>
+        <v>2.4</v>
       </c>
       <c r="P28" s="3" t="n">
-        <v>1.8</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="3" t="n">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
@@ -1951,51 +1951,51 @@
         </is>
       </c>
       <c r="C29" s="3" t="n">
-        <v>2.5</v>
+        <v>2.75</v>
       </c>
       <c r="D29" s="3" t="n">
-        <v>2.5</v>
+        <v>2</v>
       </c>
       <c r="E29" s="3" t="n">
         <v>3.75</v>
       </c>
       <c r="F29" s="3" t="n">
-        <v>1</v>
+        <v>3.5</v>
       </c>
       <c r="G29" s="3" t="n">
-        <v>3.5</v>
+        <v>4</v>
       </c>
       <c r="H29" s="3" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="I29" s="3" t="n">
-        <v>2.6</v>
+        <v>4.4</v>
       </c>
       <c r="J29" s="3" t="n">
-        <v>1.8</v>
+        <v>3.2</v>
       </c>
       <c r="K29" s="3" t="n">
-        <v>2.4</v>
+        <v>4.2</v>
       </c>
       <c r="L29" s="3" t="n">
-        <v>1</v>
+        <v>2.8</v>
       </c>
       <c r="M29" s="3" t="n">
-        <v>2.8</v>
+        <v>3</v>
       </c>
       <c r="N29" s="3" t="n">
-        <v>2.8</v>
+        <v>2.2</v>
       </c>
       <c r="O29" s="3" t="n">
-        <v>1.6</v>
+        <v>4</v>
       </c>
       <c r="P29" s="3" t="n">
-        <v>1.4</v>
+        <v>3.6</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="3" t="n">
-        <v>24</v>
+        <v>9</v>
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
@@ -2003,51 +2003,51 @@
         </is>
       </c>
       <c r="C30" s="3" t="n">
-        <v>2.75</v>
+        <v>2.5</v>
       </c>
       <c r="D30" s="3" t="n">
-        <v>3.75</v>
+        <v>2.5</v>
       </c>
       <c r="E30" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F30" s="3" t="n">
-        <v>1.25</v>
+        <v>1.5</v>
       </c>
       <c r="G30" s="3" t="n">
-        <v>3.25</v>
+        <v>3.5</v>
       </c>
       <c r="H30" s="3" t="n">
-        <v>2.75</v>
+        <v>1</v>
       </c>
       <c r="I30" s="3" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="J30" s="3" t="n">
         <v>2.8</v>
       </c>
-      <c r="J30" s="3" t="n">
+      <c r="K30" s="3" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="L30" s="3" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="M30" s="3" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="N30" s="3" t="n">
         <v>1.8</v>
       </c>
-      <c r="K30" s="3" t="n">
-        <v>3.6</v>
-      </c>
-      <c r="L30" s="3" t="n">
-        <v>1.8</v>
-      </c>
-      <c r="M30" s="3" t="n">
+      <c r="O30" s="3" t="n">
         <v>3.4</v>
       </c>
-      <c r="N30" s="3" t="n">
-        <v>3.2</v>
-      </c>
-      <c r="O30" s="3" t="n">
+      <c r="P30" s="3" t="n">
         <v>2.4</v>
-      </c>
-      <c r="P30" s="3" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="3" t="n">
-        <v>29</v>
+        <v>14</v>
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
@@ -2055,51 +2055,51 @@
         </is>
       </c>
       <c r="C31" s="3" t="n">
-        <v>2.75</v>
+        <v>3</v>
       </c>
       <c r="D31" s="3" t="n">
-        <v>2.25</v>
+        <v>3.25</v>
       </c>
       <c r="E31" s="3" t="n">
-        <v>2.75</v>
+        <v>3.5</v>
       </c>
       <c r="F31" s="3" t="n">
-        <v>1.5</v>
+        <v>3</v>
       </c>
       <c r="G31" s="3" t="n">
-        <v>2.5</v>
+        <v>3.25</v>
       </c>
       <c r="H31" s="3" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I31" s="3" t="n">
-        <v>2</v>
+        <v>3.4</v>
       </c>
       <c r="J31" s="3" t="n">
-        <v>2</v>
+        <v>2.2</v>
       </c>
       <c r="K31" s="3" t="n">
-        <v>2.6</v>
+        <v>3.6</v>
       </c>
       <c r="L31" s="3" t="n">
         <v>2</v>
       </c>
       <c r="M31" s="3" t="n">
-        <v>2.6</v>
+        <v>3.8</v>
       </c>
       <c r="N31" s="3" t="n">
-        <v>2.2</v>
+        <v>2.8</v>
       </c>
       <c r="O31" s="3" t="n">
-        <v>2.2</v>
+        <v>2.8</v>
       </c>
       <c r="P31" s="3" t="n">
-        <v>2</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="3" t="n">
-        <v>34</v>
+        <v>19</v>
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
@@ -2110,48 +2110,48 @@
         <v>2.5</v>
       </c>
       <c r="D32" s="3" t="n">
-        <v>2</v>
+        <v>2.5</v>
       </c>
       <c r="E32" s="3" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="F32" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G32" s="3" t="n">
         <v>3.5</v>
       </c>
-      <c r="F32" s="3" t="n">
-        <v>3.5</v>
-      </c>
-      <c r="G32" s="3" t="n">
-        <v>3</v>
-      </c>
       <c r="H32" s="3" t="n">
-        <v>2.75</v>
+        <v>1</v>
       </c>
       <c r="I32" s="3" t="n">
         <v>2.6</v>
       </c>
       <c r="J32" s="3" t="n">
-        <v>3.4</v>
+        <v>1.8</v>
       </c>
       <c r="K32" s="3" t="n">
-        <v>4</v>
+        <v>2.4</v>
       </c>
       <c r="L32" s="3" t="n">
-        <v>2.4</v>
+        <v>1</v>
       </c>
       <c r="M32" s="3" t="n">
-        <v>3.8</v>
+        <v>2.8</v>
       </c>
       <c r="N32" s="3" t="n">
-        <v>1.8</v>
+        <v>2.8</v>
       </c>
       <c r="O32" s="3" t="n">
         <v>1.6</v>
       </c>
       <c r="P32" s="3" t="n">
-        <v>1</v>
+        <v>1.4</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="3" t="n">
-        <v>39</v>
+        <v>24</v>
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
@@ -2159,43 +2159,43 @@
         </is>
       </c>
       <c r="C33" s="3" t="n">
-        <v>2</v>
+        <v>2.75</v>
       </c>
       <c r="D33" s="3" t="n">
-        <v>2</v>
+        <v>3.75</v>
       </c>
       <c r="E33" s="3" t="n">
-        <v>3.5</v>
+        <v>3</v>
       </c>
       <c r="F33" s="3" t="n">
-        <v>3</v>
+        <v>1.25</v>
       </c>
       <c r="G33" s="3" t="n">
-        <v>3</v>
+        <v>3.25</v>
       </c>
       <c r="H33" s="3" t="n">
-        <v>3</v>
+        <v>2.75</v>
       </c>
       <c r="I33" s="3" t="n">
-        <v>1.8</v>
+        <v>2.8</v>
       </c>
       <c r="J33" s="3" t="n">
         <v>1.8</v>
       </c>
       <c r="K33" s="3" t="n">
-        <v>2.2</v>
+        <v>3.6</v>
       </c>
       <c r="L33" s="3" t="n">
-        <v>2.8</v>
+        <v>1.8</v>
       </c>
       <c r="M33" s="3" t="n">
-        <v>1</v>
+        <v>3.4</v>
       </c>
       <c r="N33" s="3" t="n">
-        <v>1</v>
+        <v>3.2</v>
       </c>
       <c r="O33" s="3" t="n">
-        <v>1.8</v>
+        <v>2.4</v>
       </c>
       <c r="P33" s="3" t="n">
         <v>1</v>
@@ -2203,155 +2203,155 @@
     </row>
     <row r="34">
       <c r="A34" s="3" t="n">
-        <v>5</v>
+        <v>29</v>
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>II</t>
+          <t>CI</t>
         </is>
       </c>
       <c r="C34" s="3" t="n">
         <v>2.75</v>
       </c>
       <c r="D34" s="3" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="E34" s="3" t="n">
         <v>2.75</v>
       </c>
-      <c r="E34" s="3" t="n">
-        <v>4</v>
-      </c>
       <c r="F34" s="3" t="n">
-        <v>4</v>
+        <v>1.5</v>
       </c>
       <c r="G34" s="3" t="n">
-        <v>1.75</v>
+        <v>2.5</v>
       </c>
       <c r="H34" s="3" t="n">
-        <v>1.5</v>
+        <v>1</v>
       </c>
       <c r="I34" s="3" t="n">
-        <v>2.8</v>
+        <v>2</v>
       </c>
       <c r="J34" s="3" t="n">
-        <v>2.8</v>
+        <v>2</v>
       </c>
       <c r="K34" s="3" t="n">
-        <v>3.2</v>
+        <v>2.6</v>
       </c>
       <c r="L34" s="3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M34" s="3" t="n">
-        <v>3.8</v>
+        <v>2.6</v>
       </c>
       <c r="N34" s="3" t="n">
-        <v>3</v>
+        <v>2.2</v>
       </c>
       <c r="O34" s="3" t="n">
-        <v>2.6</v>
+        <v>2.2</v>
       </c>
       <c r="P34" s="3" t="n">
-        <v>2.2</v>
+        <v>2</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="3" t="n">
-        <v>10</v>
+        <v>34</v>
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>II</t>
+          <t>CI</t>
         </is>
       </c>
       <c r="C35" s="3" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="D35" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="D35" s="3" t="n">
-        <v>1.25</v>
-      </c>
       <c r="E35" s="3" t="n">
-        <v>1</v>
+        <v>3.5</v>
       </c>
       <c r="F35" s="3" t="n">
-        <v>1.25</v>
+        <v>3.5</v>
       </c>
       <c r="G35" s="3" t="n">
-        <v>1.25</v>
+        <v>3</v>
       </c>
       <c r="H35" s="3" t="n">
-        <v>1.5</v>
+        <v>2.75</v>
       </c>
       <c r="I35" s="3" t="n">
-        <v>2.2</v>
+        <v>2.6</v>
       </c>
       <c r="J35" s="3" t="n">
-        <v>1.8</v>
+        <v>3.4</v>
       </c>
       <c r="K35" s="3" t="n">
-        <v>1.6</v>
+        <v>4</v>
       </c>
       <c r="L35" s="3" t="n">
-        <v>1.4</v>
+        <v>2.4</v>
       </c>
       <c r="M35" s="3" t="n">
-        <v>1.6</v>
+        <v>3.8</v>
       </c>
       <c r="N35" s="3" t="n">
         <v>1.8</v>
       </c>
       <c r="O35" s="3" t="n">
-        <v>1.2</v>
+        <v>1.6</v>
       </c>
       <c r="P35" s="3" t="n">
-        <v>1.6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="3" t="n">
-        <v>15</v>
+        <v>39</v>
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>II</t>
+          <t>CI</t>
         </is>
       </c>
       <c r="C36" s="3" t="n">
-        <v>1.75</v>
+        <v>2</v>
       </c>
       <c r="D36" s="3" t="n">
-        <v>1.75</v>
+        <v>2</v>
       </c>
       <c r="E36" s="3" t="n">
-        <v>1</v>
+        <v>3.5</v>
       </c>
       <c r="F36" s="3" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G36" s="3" t="n">
-        <v>1.75</v>
+        <v>3</v>
       </c>
       <c r="H36" s="3" t="n">
-        <v>1.5</v>
+        <v>3</v>
       </c>
       <c r="I36" s="3" t="n">
-        <v>1.4</v>
+        <v>1.8</v>
       </c>
       <c r="J36" s="3" t="n">
-        <v>1.2</v>
+        <v>1.8</v>
       </c>
       <c r="K36" s="3" t="n">
-        <v>2</v>
+        <v>2.2</v>
       </c>
       <c r="L36" s="3" t="n">
-        <v>1.6</v>
+        <v>2.8</v>
       </c>
       <c r="M36" s="3" t="n">
-        <v>2.2</v>
+        <v>1</v>
       </c>
       <c r="N36" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O36" s="3" t="n">
-        <v>1.2</v>
+        <v>1.8</v>
       </c>
       <c r="P36" s="3" t="n">
         <v>1</v>
@@ -2359,59 +2359,59 @@
     </row>
     <row r="37">
       <c r="A37" s="3" t="n">
-        <v>20</v>
+        <v>44</v>
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>II</t>
+          <t>CI</t>
         </is>
       </c>
       <c r="C37" s="3" t="n">
-        <v>3</v>
+        <v>1.25</v>
       </c>
       <c r="D37" s="3" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E37" s="3" t="n">
-        <v>3.25</v>
+        <v>3.75</v>
       </c>
       <c r="F37" s="3" t="n">
-        <v>3</v>
+        <v>1.75</v>
       </c>
       <c r="G37" s="3" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H37" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I37" s="3" t="n">
-        <v>1.8</v>
+        <v>3.4</v>
       </c>
       <c r="J37" s="3" t="n">
-        <v>2.6</v>
+        <v>1.2</v>
       </c>
       <c r="K37" s="3" t="n">
-        <v>2.8</v>
+        <v>3.8</v>
       </c>
       <c r="L37" s="3" t="n">
-        <v>3.2</v>
+        <v>1</v>
       </c>
       <c r="M37" s="3" t="n">
-        <v>2.8</v>
+        <v>1</v>
       </c>
       <c r="N37" s="3" t="n">
-        <v>2.4</v>
+        <v>1</v>
       </c>
       <c r="O37" s="3" t="n">
-        <v>2.6</v>
+        <v>1.4</v>
       </c>
       <c r="P37" s="3" t="n">
-        <v>2.8</v>
+        <v>1</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="3" t="n">
-        <v>25</v>
+        <v>5</v>
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
@@ -2419,51 +2419,51 @@
         </is>
       </c>
       <c r="C38" s="3" t="n">
-        <v>2</v>
+        <v>2.75</v>
       </c>
       <c r="D38" s="3" t="n">
-        <v>2</v>
+        <v>2.75</v>
       </c>
       <c r="E38" s="3" t="n">
-        <v>2.5</v>
+        <v>4</v>
       </c>
       <c r="F38" s="3" t="n">
-        <v>2.25</v>
+        <v>4</v>
       </c>
       <c r="G38" s="3" t="n">
-        <v>1</v>
+        <v>1.75</v>
       </c>
       <c r="H38" s="3" t="n">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="I38" s="3" t="n">
-        <v>1.8</v>
+        <v>2.8</v>
       </c>
       <c r="J38" s="3" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="K38" s="3" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="L38" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="M38" s="3" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="N38" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="O38" s="3" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="P38" s="3" t="n">
         <v>2.2</v>
-      </c>
-      <c r="K38" s="3" t="n">
-        <v>2.8</v>
-      </c>
-      <c r="L38" s="3" t="n">
-        <v>2.2</v>
-      </c>
-      <c r="M38" s="3" t="n">
-        <v>1.8</v>
-      </c>
-      <c r="N38" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="O38" s="3" t="n">
-        <v>3.4</v>
-      </c>
-      <c r="P38" s="3" t="n">
-        <v>2</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="3" t="n">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
@@ -2471,51 +2471,51 @@
         </is>
       </c>
       <c r="C39" s="3" t="n">
-        <v>3.75</v>
+        <v>2</v>
       </c>
       <c r="D39" s="3" t="n">
-        <v>3.75</v>
+        <v>1.25</v>
       </c>
       <c r="E39" s="3" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F39" s="3" t="n">
-        <v>3.75</v>
+        <v>1.25</v>
       </c>
       <c r="G39" s="3" t="n">
-        <v>3.5</v>
+        <v>1.25</v>
       </c>
       <c r="H39" s="3" t="n">
-        <v>3</v>
+        <v>1.5</v>
       </c>
       <c r="I39" s="3" t="n">
-        <v>2.8</v>
+        <v>2.2</v>
       </c>
       <c r="J39" s="3" t="n">
-        <v>3.4</v>
+        <v>1.8</v>
       </c>
       <c r="K39" s="3" t="n">
-        <v>3.4</v>
+        <v>1.6</v>
       </c>
       <c r="L39" s="3" t="n">
-        <v>3.8</v>
+        <v>1.4</v>
       </c>
       <c r="M39" s="3" t="n">
-        <v>2.8</v>
+        <v>1.6</v>
       </c>
       <c r="N39" s="3" t="n">
-        <v>4.2</v>
+        <v>1.8</v>
       </c>
       <c r="O39" s="3" t="n">
-        <v>2</v>
+        <v>1.2</v>
       </c>
       <c r="P39" s="3" t="n">
-        <v>2.2</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="3" t="n">
-        <v>35</v>
+        <v>15</v>
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
@@ -2523,98 +2523,358 @@
         </is>
       </c>
       <c r="C40" s="3" t="n">
-        <v>2.5</v>
+        <v>1.75</v>
       </c>
       <c r="D40" s="3" t="n">
-        <v>2</v>
+        <v>1.75</v>
       </c>
       <c r="E40" s="3" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F40" s="3" t="n">
-        <v>3.25</v>
+        <v>1</v>
       </c>
       <c r="G40" s="3" t="n">
-        <v>1</v>
+        <v>1.75</v>
       </c>
       <c r="H40" s="3" t="n">
         <v>1.5</v>
       </c>
       <c r="I40" s="3" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="J40" s="3" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="K40" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="J40" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="K40" s="3" t="n">
+      <c r="L40" s="3" t="n">
         <v>1.6</v>
       </c>
-      <c r="L40" s="3" t="n">
-        <v>1</v>
-      </c>
       <c r="M40" s="3" t="n">
-        <v>1.4</v>
+        <v>2.2</v>
       </c>
       <c r="N40" s="3" t="n">
-        <v>2.8</v>
+        <v>2</v>
       </c>
       <c r="O40" s="3" t="n">
-        <v>2.8</v>
+        <v>1.2</v>
       </c>
       <c r="P40" s="3" t="n">
-        <v>1.4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="B41" s="3" t="inlineStr">
+        <is>
+          <t>II</t>
+        </is>
+      </c>
+      <c r="C41" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="D41" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E41" s="3" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="F41" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="G41" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="H41" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="I41" s="3" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="J41" s="3" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="K41" s="3" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="L41" s="3" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="M41" s="3" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="N41" s="3" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="O41" s="3" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="P41" s="3" t="n">
+        <v>2.8</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="3" t="n">
+        <v>25</v>
+      </c>
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>II</t>
+        </is>
+      </c>
+      <c r="C42" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D42" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E42" s="3" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F42" s="3" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="G42" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="H42" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="I42" s="3" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="J42" s="3" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="K42" s="3" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="L42" s="3" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="M42" s="3" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="N42" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="O42" s="3" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="P42" s="3" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="B43" s="3" t="inlineStr">
+        <is>
+          <t>II</t>
+        </is>
+      </c>
+      <c r="C43" s="3" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="D43" s="3" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="E43" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="F43" s="3" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="G43" s="3" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="H43" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="I43" s="3" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="J43" s="3" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="K43" s="3" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="L43" s="3" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="M43" s="3" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="N43" s="3" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="O43" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="P43" s="3" t="n">
+        <v>2.2</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="3" t="n">
+        <v>35</v>
+      </c>
+      <c r="B44" s="3" t="inlineStr">
+        <is>
+          <t>II</t>
+        </is>
+      </c>
+      <c r="C44" s="3" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="D44" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E44" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="F44" s="3" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="G44" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="H44" s="3" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="I44" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="J44" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="K44" s="3" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="L44" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="M44" s="3" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="N44" s="3" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="O44" s="3" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="P44" s="3" t="n">
+        <v>1.4</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="3" t="n">
         <v>40</v>
       </c>
-      <c r="B41" s="3" t="inlineStr">
+      <c r="B45" s="3" t="inlineStr">
         <is>
           <t>II</t>
         </is>
       </c>
-      <c r="C41" s="3" t="n">
+      <c r="C45" s="3" t="n">
         <v>2.25</v>
       </c>
-      <c r="D41" s="3" t="n">
+      <c r="D45" s="3" t="n">
         <v>2.25</v>
       </c>
-      <c r="E41" s="3" t="n">
+      <c r="E45" s="3" t="n">
         <v>1.75</v>
       </c>
-      <c r="F41" s="3" t="n">
+      <c r="F45" s="3" t="n">
         <v>2.25</v>
       </c>
-      <c r="G41" s="3" t="n">
+      <c r="G45" s="3" t="n">
         <v>1.75</v>
       </c>
-      <c r="H41" s="3" t="n">
+      <c r="H45" s="3" t="n">
         <v>1.75</v>
       </c>
-      <c r="I41" s="3" t="n">
+      <c r="I45" s="3" t="n">
         <v>2.2</v>
       </c>
-      <c r="J41" s="3" t="n">
+      <c r="J45" s="3" t="n">
         <v>1.8</v>
       </c>
-      <c r="K41" s="3" t="n">
+      <c r="K45" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="L41" s="3" t="n">
+      <c r="L45" s="3" t="n">
         <v>1.4</v>
       </c>
-      <c r="M41" s="3" t="n">
+      <c r="M45" s="3" t="n">
         <v>3.2</v>
       </c>
-      <c r="N41" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="O41" s="3" t="n">
+      <c r="N45" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="O45" s="3" t="n">
         <v>1.6</v>
       </c>
-      <c r="P41" s="3" t="n">
+      <c r="P45" s="3" t="n">
         <v>1.6</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="3" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" s="3" t="inlineStr">
+        <is>
+          <t>II</t>
+        </is>
+      </c>
+      <c r="C46" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D46" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E46" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F46" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="G46" s="3" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="H46" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="I46" s="3" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="J46" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="K46" s="3" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="L46" s="3" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="M46" s="3" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="N46" s="3" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="O46" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="P46" s="3" t="n">
+        <v>3</v>
       </c>
     </row>
   </sheetData>
@@ -2635,7 +2895,7 @@
     <col width="23" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="23" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
     <col width="25" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -2684,14 +2944,14 @@
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>ANOVA</t>
+          <t>Kruskal-Wallis</t>
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>0.979238682212762</v>
+        <v>8.199202279202282</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>0.431403539796531</v>
+        <v>0.08454775039006411</v>
       </c>
       <c r="F2" s="3" t="b">
         <v>0</v>
@@ -2714,10 +2974,10 @@
         </is>
       </c>
       <c r="D3" s="3" t="n">
-        <v>1.338038719612804</v>
+        <v>1.852134793311265</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>0.2753019020930046</v>
+        <v>0.1378906198067127</v>
       </c>
       <c r="F3" s="3" t="b">
         <v>0</v>
@@ -2740,13 +3000,13 @@
         </is>
       </c>
       <c r="D4" s="3" t="n">
-        <v>9.205523451845574</v>
+        <v>11.61249786167452</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>0.05616272016762326</v>
+        <v>0.02047792545214611</v>
       </c>
       <c r="F4" s="3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5">
@@ -2766,13 +3026,13 @@
         </is>
       </c>
       <c r="D5" s="3" t="n">
-        <v>8.461582456999572</v>
+        <v>9.849176048295007</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>0.07606031193307826</v>
+        <v>0.04304639156140955</v>
       </c>
       <c r="F5" s="3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6">
@@ -2792,10 +3052,10 @@
         </is>
       </c>
       <c r="D6" s="3" t="n">
-        <v>17.39210567666436</v>
+        <v>19.76245333333334</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>0.001621612978210302</v>
+        <v>0.0005563084304493354</v>
       </c>
       <c r="F6" s="3" t="b">
         <v>1</v>
@@ -2818,10 +3078,10 @@
         </is>
       </c>
       <c r="D7" s="3" t="n">
-        <v>12.0904833736041</v>
+        <v>13.98984766308051</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>0.01669093976383364</v>
+        <v>0.007327528379958215</v>
       </c>
       <c r="F7" s="3" t="b">
         <v>1</v>
@@ -2848,14 +3108,14 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>T-test</t>
+          <t>Wilcoxon</t>
         </is>
       </c>
       <c r="D9" s="3" t="n">
-        <v>-0.25</v>
+        <v>10.5</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>0.8088874454935351</v>
+        <v>0.328125</v>
       </c>
       <c r="F9" s="3" t="b">
         <v>0</v>
@@ -2904,10 +3164,10 @@
         </is>
       </c>
       <c r="D11" s="3" t="n">
-        <v>-1.276939015148195</v>
+        <v>-1.075862591114976</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>0.2374378627385179</v>
+        <v>0.3099823248900485</v>
       </c>
       <c r="F11" s="3" t="b">
         <v>0</v>
@@ -2941,7 +3201,7 @@
         <v>1</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="F13" s="3" t="b">
         <v>0</v>
@@ -2964,10 +3224,10 @@
         </is>
       </c>
       <c r="D14" s="3" t="n">
-        <v>1.692228224453299</v>
+        <v>2.186844946600275</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>0.1415500090567489</v>
+        <v>0.06498072941386071</v>
       </c>
       <c r="F14" s="3" t="b">
         <v>0</v>
@@ -2990,13 +3250,13 @@
         </is>
       </c>
       <c r="D15" s="3" t="n">
-        <v>2.208193696890079</v>
+        <v>2.737804817958895</v>
       </c>
       <c r="E15" s="3" t="n">
-        <v>0.06931549051135975</v>
+        <v>0.02900994379056727</v>
       </c>
       <c r="F15" s="3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16">
@@ -3020,14 +3280,14 @@
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>T-test</t>
+          <t>Wilcoxon</t>
         </is>
       </c>
       <c r="D17" s="3" t="n">
-        <v>1.210419877178893</v>
+        <v>7.5</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>0.2653980394260696</v>
+        <v>0.1796875</v>
       </c>
       <c r="F17" s="3" t="b">
         <v>0</v>
@@ -3050,10 +3310,10 @@
         </is>
       </c>
       <c r="D18" s="3" t="n">
-        <v>1.029472235716996</v>
+        <v>1.422656703427915</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>0.3375098903355412</v>
+        <v>0.1926360712795102</v>
       </c>
       <c r="F18" s="3" t="b">
         <v>0</v>
@@ -3079,7 +3339,7 @@
         <v>0</v>
       </c>
       <c r="E19" s="3" t="n">
-        <v>0.125</v>
+        <v>0.0625</v>
       </c>
       <c r="F19" s="3" t="b">
         <v>0</v>
@@ -3110,10 +3370,10 @@
         </is>
       </c>
       <c r="D21" s="3" t="n">
-        <v>0.3232299675777271</v>
+        <v>0.4850712500726659</v>
       </c>
       <c r="E21" s="3" t="n">
-        <v>0.7559627503969001</v>
+        <v>0.6406295692605111</v>
       </c>
       <c r="F21" s="3" t="b">
         <v>0</v>
@@ -3136,10 +3396,10 @@
         </is>
       </c>
       <c r="D22" s="3" t="n">
-        <v>3.198557367121814</v>
+        <v>3.76215977250384</v>
       </c>
       <c r="E22" s="3" t="n">
-        <v>0.015096034879553</v>
+        <v>0.005527234779639096</v>
       </c>
       <c r="F22" s="3" t="b">
         <v>1</v>
@@ -3162,10 +3422,10 @@
         </is>
       </c>
       <c r="D23" s="3" t="n">
-        <v>1.846407837401394</v>
+        <v>2.304092101743771</v>
       </c>
       <c r="E23" s="3" t="n">
-        <v>0.1073313153411767</v>
+        <v>0.05014946025596994</v>
       </c>
       <c r="F23" s="3" t="b">
         <v>0</v>
@@ -3222,10 +3482,10 @@
         </is>
       </c>
       <c r="D26" s="3" t="n">
-        <v>-0.3139929128113796</v>
+        <v>-1</v>
       </c>
       <c r="E26" s="3" t="n">
-        <v>0.7626770646286338</v>
+        <v>0.3465935070873342</v>
       </c>
       <c r="F26" s="3" t="b">
         <v>0</v>
@@ -3248,10 +3508,10 @@
         </is>
       </c>
       <c r="D27" s="3" t="n">
-        <v>-0.5516772843673705</v>
+        <v>-0.3592106040535498</v>
       </c>
       <c r="E27" s="3" t="n">
-        <v>0.5983311559987459</v>
+        <v>0.7287339886104589</v>
       </c>
       <c r="F27" s="3" t="b">
         <v>0</v>
@@ -3276,12 +3536,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:F41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="23" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
@@ -3331,15 +3591,15 @@
         </is>
       </c>
       <c r="C2" s="3" t="n">
-        <v>0.9608018940605703</v>
+        <v>0.01763157110729855</v>
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>TRU_D</t>
+          <t>HLP_D</t>
         </is>
       </c>
       <c r="E2" s="3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
@@ -3359,15 +3619,15 @@
         </is>
       </c>
       <c r="C3" s="3" t="n">
-        <v>0.04784722458896093</v>
+        <v>0.1739208752908169</v>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>TRU_D</t>
+          <t>HLP_D</t>
         </is>
       </c>
       <c r="E3" s="3" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
@@ -3387,11 +3647,11 @@
         </is>
       </c>
       <c r="C4" s="3" t="n">
-        <v>0.6263814204856222</v>
+        <v>0.8686158872054418</v>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>TRU_D</t>
+          <t>HLP_D</t>
         </is>
       </c>
       <c r="E4" s="3" t="b">
@@ -3415,11 +3675,11 @@
         </is>
       </c>
       <c r="C5" s="3" t="n">
-        <v>0.00488110702362953</v>
+        <v>0.008929369627695161</v>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>TRU_D</t>
+          <t>HLP_D</t>
         </is>
       </c>
       <c r="E5" s="3" t="b">
@@ -3443,15 +3703,15 @@
         </is>
       </c>
       <c r="C6" s="3" t="n">
-        <v>0.02938892047286141</v>
+        <v>0.9222904004085215</v>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>TRU_D</t>
+          <t>HLP_D</t>
         </is>
       </c>
       <c r="E6" s="3" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
@@ -3471,11 +3731,11 @@
         </is>
       </c>
       <c r="C7" s="3" t="n">
-        <v>0.4572444216238805</v>
+        <v>0.2108731475949404</v>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>TRU_D</t>
+          <t>HLP_D</t>
         </is>
       </c>
       <c r="E7" s="3" t="b">
@@ -3499,15 +3759,15 @@
         </is>
       </c>
       <c r="C8" s="3" t="n">
-        <v>0.006809150097497262</v>
+        <v>0.08283519531275839</v>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>TRU_D</t>
+          <t>HLP_D</t>
         </is>
       </c>
       <c r="E8" s="3" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
@@ -3527,11 +3787,11 @@
         </is>
       </c>
       <c r="C9" s="3" t="n">
-        <v>0.558947374068095</v>
+        <v>0.3582775113547582</v>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>TRU_D</t>
+          <t>HLP_D</t>
         </is>
       </c>
       <c r="E9" s="3" t="b">
@@ -3555,15 +3815,15 @@
         </is>
       </c>
       <c r="C10" s="3" t="n">
-        <v>0.002827330717951227</v>
+        <v>0.09851354799126623</v>
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>TRU_D</t>
+          <t>HLP_D</t>
         </is>
       </c>
       <c r="E10" s="3" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
@@ -3583,11 +3843,11 @@
         </is>
       </c>
       <c r="C11" s="3" t="n">
-        <v>0.003544521685164924</v>
+        <v>0.0188489323303409</v>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>TRU_D</t>
+          <t>HLP_D</t>
         </is>
       </c>
       <c r="E11" s="3" t="b">
@@ -3611,15 +3871,15 @@
         </is>
       </c>
       <c r="C12" s="3" t="n">
-        <v>0.05651855511195005</v>
+        <v>0.02137009205072758</v>
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>TRU_M</t>
+          <t>HLP_M</t>
         </is>
       </c>
       <c r="E12" s="3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
@@ -3639,11 +3899,11 @@
         </is>
       </c>
       <c r="C13" s="3" t="n">
-        <v>0.2873273855988826</v>
+        <v>0.09337047157937436</v>
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>TRU_M</t>
+          <t>HLP_M</t>
         </is>
       </c>
       <c r="E13" s="3" t="b">
@@ -3667,11 +3927,11 @@
         </is>
       </c>
       <c r="C14" s="3" t="n">
-        <v>0.4936154695260365</v>
+        <v>0.8689660310637081</v>
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>TRU_M</t>
+          <t>HLP_M</t>
         </is>
       </c>
       <c r="E14" s="3" t="b">
@@ -3695,15 +3955,15 @@
         </is>
       </c>
       <c r="C15" s="3" t="n">
-        <v>0.001522588585183457</v>
+        <v>0.05735653368808483</v>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>TRU_M</t>
+          <t>HLP_M</t>
         </is>
       </c>
       <c r="E15" s="3" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
@@ -3723,11 +3983,11 @@
         </is>
       </c>
       <c r="C16" s="3" t="n">
-        <v>0.7256159408473616</v>
+        <v>0.5270748756635324</v>
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>TRU_M</t>
+          <t>HLP_M</t>
         </is>
       </c>
       <c r="E16" s="3" t="b">
@@ -3751,15 +4011,15 @@
         </is>
       </c>
       <c r="C17" s="3" t="n">
-        <v>0.2622863556732082</v>
+        <v>0.02609189888140067</v>
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>TRU_M</t>
+          <t>HLP_M</t>
         </is>
       </c>
       <c r="E17" s="3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
@@ -3779,11 +4039,11 @@
         </is>
       </c>
       <c r="C18" s="3" t="n">
-        <v>0.5208480313753976</v>
+        <v>0.4764962391065515</v>
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>TRU_M</t>
+          <t>HLP_M</t>
         </is>
       </c>
       <c r="E18" s="3" t="b">
@@ -3807,11 +4067,11 @@
         </is>
       </c>
       <c r="C19" s="3" t="n">
-        <v>0.3200302155933907</v>
+        <v>0.1201964415000216</v>
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>TRU_M</t>
+          <t>HLP_M</t>
         </is>
       </c>
       <c r="E19" s="3" t="b">
@@ -3835,11 +4095,11 @@
         </is>
       </c>
       <c r="C20" s="3" t="n">
-        <v>0.1985503644638253</v>
+        <v>1</v>
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>TRU_M</t>
+          <t>HLP_M</t>
         </is>
       </c>
       <c r="E20" s="3" t="b">
@@ -3863,17 +4123,577 @@
         </is>
       </c>
       <c r="C21" s="3" t="n">
-        <v>0.00402709286994327</v>
+        <v>0.1095521838076782</v>
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
+          <t>HLP_M</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>Holm</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>CC</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>CI</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="n">
+        <v>0.6764477161764175</v>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>TRU_D</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>Holm</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>CC</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>CS0</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="n">
+        <v>0.08869784561484315</v>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>TRU_D</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="F23" s="3" t="inlineStr">
+        <is>
+          <t>Holm</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>CC</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>CS1</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="n">
+        <v>0.9012656769084249</v>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>TRU_D</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>Holm</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>CC</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>II</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="n">
+        <v>0.002367665798685567</v>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>TRU_D</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="F25" s="3" t="inlineStr">
+        <is>
+          <t>Holm</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>CI</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>CS0</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="n">
+        <v>0.01286443677409298</v>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>TRU_D</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="F26" s="3" t="inlineStr">
+        <is>
+          <t>Holm</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>CI</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>CS1</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="n">
+        <v>0.5596433018488416</v>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>TRU_D</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="F27" s="3" t="inlineStr">
+        <is>
+          <t>Holm</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>CI</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>II</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="n">
+        <v>0.003283460986069043</v>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>TRU_D</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="F28" s="3" t="inlineStr">
+        <is>
+          <t>Holm</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>CS0</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>CS1</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="n">
+        <v>0.3829551122087131</v>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>TRU_D</t>
+        </is>
+      </c>
+      <c r="E29" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="F29" s="3" t="inlineStr">
+        <is>
+          <t>Holm</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>CS0</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>II</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="n">
+        <v>0.001155968418808117</v>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>TRU_D</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="F30" s="3" t="inlineStr">
+        <is>
+          <t>Holm</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>CS1</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>II</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="n">
+        <v>0.001851041013977846</v>
+      </c>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>TRU_D</t>
+        </is>
+      </c>
+      <c r="E31" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="F31" s="3" t="inlineStr">
+        <is>
+          <t>Holm</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="inlineStr">
+        <is>
+          <t>CC</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>CI</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="n">
+        <v>0.02269160738446154</v>
+      </c>
+      <c r="D32" s="3" t="inlineStr">
+        <is>
           <t>TRU_M</t>
         </is>
       </c>
-      <c r="E21" s="3" t="b">
-        <v>1</v>
-      </c>
-      <c r="F21" s="3" t="inlineStr">
+      <c r="E32" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="F32" s="3" t="inlineStr">
+        <is>
+          <t>Holm</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t>CC</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>CS0</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="n">
+        <v>0.1287280653570155</v>
+      </c>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>TRU_M</t>
+        </is>
+      </c>
+      <c r="E33" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="F33" s="3" t="inlineStr">
+        <is>
+          <t>Holm</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>CC</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>CS1</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="n">
+        <v>0.3211708098118675</v>
+      </c>
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>TRU_M</t>
+        </is>
+      </c>
+      <c r="E34" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="F34" s="3" t="inlineStr">
+        <is>
+          <t>Holm</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
+          <t>CC</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>II</t>
+        </is>
+      </c>
+      <c r="C35" s="3" t="n">
+        <v>0.0007079635731724508</v>
+      </c>
+      <c r="D35" s="3" t="inlineStr">
+        <is>
+          <t>TRU_M</t>
+        </is>
+      </c>
+      <c r="E35" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="F35" s="3" t="inlineStr">
+        <is>
+          <t>Holm</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="3" t="inlineStr">
+        <is>
+          <t>CI</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>CS0</t>
+        </is>
+      </c>
+      <c r="C36" s="3" t="n">
+        <v>0.730325149398968</v>
+      </c>
+      <c r="D36" s="3" t="inlineStr">
+        <is>
+          <t>TRU_M</t>
+        </is>
+      </c>
+      <c r="E36" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="F36" s="3" t="inlineStr">
+        <is>
+          <t>Holm</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="3" t="inlineStr">
+        <is>
+          <t>CI</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="inlineStr">
+        <is>
+          <t>CS1</t>
+        </is>
+      </c>
+      <c r="C37" s="3" t="n">
+        <v>0.2094225501070196</v>
+      </c>
+      <c r="D37" s="3" t="inlineStr">
+        <is>
+          <t>TRU_M</t>
+        </is>
+      </c>
+      <c r="E37" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="F37" s="3" t="inlineStr">
+        <is>
+          <t>Holm</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="3" t="inlineStr">
+        <is>
+          <t>CI</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>II</t>
+        </is>
+      </c>
+      <c r="C38" s="3" t="n">
+        <v>0.7871842287447913</v>
+      </c>
+      <c r="D38" s="3" t="inlineStr">
+        <is>
+          <t>TRU_M</t>
+        </is>
+      </c>
+      <c r="E38" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="F38" s="3" t="inlineStr">
+        <is>
+          <t>Holm</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="3" t="inlineStr">
+        <is>
+          <t>CS0</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="inlineStr">
+        <is>
+          <t>CS1</t>
+        </is>
+      </c>
+      <c r="C39" s="3" t="n">
+        <v>0.2064551948012603</v>
+      </c>
+      <c r="D39" s="3" t="inlineStr">
+        <is>
+          <t>TRU_M</t>
+        </is>
+      </c>
+      <c r="E39" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="F39" s="3" t="inlineStr">
+        <is>
+          <t>Holm</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="3" t="inlineStr">
+        <is>
+          <t>CS0</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>II</t>
+        </is>
+      </c>
+      <c r="C40" s="3" t="n">
+        <v>0.4090675120734073</v>
+      </c>
+      <c r="D40" s="3" t="inlineStr">
+        <is>
+          <t>TRU_M</t>
+        </is>
+      </c>
+      <c r="E40" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="F40" s="3" t="inlineStr">
+        <is>
+          <t>Holm</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="3" t="inlineStr">
+        <is>
+          <t>CS1</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="inlineStr">
+        <is>
+          <t>II</t>
+        </is>
+      </c>
+      <c r="C41" s="3" t="n">
+        <v>0.00237718751242023</v>
+      </c>
+      <c r="D41" s="3" t="inlineStr">
+        <is>
+          <t>TRU_M</t>
+        </is>
+      </c>
+      <c r="E41" s="3" t="b">
+        <v>1</v>
+      </c>
+      <c r="F41" s="3" t="inlineStr">
         <is>
           <t>Holm</t>
         </is>
@@ -3896,7 +4716,7 @@
     <col width="17" customWidth="1" min="1" max="1"/>
     <col width="23" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
     <col width="23" customWidth="1" min="5" max="5"/>
     <col width="25" customWidth="1" min="6" max="6"/>
   </cols>
@@ -3950,10 +4770,10 @@
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>3.95670387914768</v>
+        <v>3.393329208616907</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>0.009420541846232398</v>
+        <v>0.01758801924811175</v>
       </c>
       <c r="F2" s="3" t="b">
         <v>1</v>
@@ -3976,13 +4796,13 @@
         </is>
       </c>
       <c r="D3" s="3" t="n">
-        <v>2.257194392720053</v>
+        <v>2.663619635543421</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>0.08269593347326513</v>
+        <v>0.04628152591003986</v>
       </c>
       <c r="F3" s="3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4">
@@ -4002,10 +4822,10 @@
         </is>
       </c>
       <c r="D4" s="3" t="n">
-        <v>2.708393082524991</v>
+        <v>3.216141407274316</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>0.04582870018036539</v>
+        <v>0.0221984071626053</v>
       </c>
       <c r="F4" s="3" t="b">
         <v>1</v>
@@ -4028,10 +4848,10 @@
         </is>
       </c>
       <c r="D5" s="3" t="n">
-        <v>3.178952996463713</v>
+        <v>3.68323966844111</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>0.02498570255569007</v>
+        <v>0.01205828426346624</v>
       </c>
       <c r="F5" s="3" t="b">
         <v>1</v>
@@ -4054,10 +4874,10 @@
         </is>
       </c>
       <c r="D6" s="3" t="n">
-        <v>1.878348101265823</v>
+        <v>2.071446756622761</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>0.1361469280875903</v>
+        <v>0.1026623249159224</v>
       </c>
       <c r="F6" s="3" t="b">
         <v>0</v>
@@ -4080,10 +4900,10 @@
         </is>
       </c>
       <c r="D7" s="3" t="n">
-        <v>1.339111507726844</v>
+        <v>1.853853787428626</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>0.2749236113576879</v>
+        <v>0.1375728005606608</v>
       </c>
       <c r="F7" s="3" t="b">
         <v>0</v>
@@ -4106,10 +4926,10 @@
         </is>
       </c>
       <c r="D8" s="3" t="n">
-        <v>3.11234964218647</v>
+        <v>2.98901643521023</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>0.02720711948876369</v>
+        <v>0.02998105243280189</v>
       </c>
       <c r="F8" s="3" t="b">
         <v>1</v>
@@ -4128,14 +4948,14 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>ANOVA</t>
+          <t>Kruskal-Wallis</t>
         </is>
       </c>
       <c r="D9" s="3" t="n">
-        <v>4.020055095788944</v>
+        <v>11.77810761009765</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>0.008715363880588878</v>
+        <v>0.01907989610544843</v>
       </c>
       <c r="F9" s="3" t="b">
         <v>1</v>
@@ -4166,10 +4986,10 @@
         </is>
       </c>
       <c r="D11" s="3" t="n">
-        <v>-1.091089451179962</v>
+        <v>-1.16968842918859</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>0.3070016039744494</v>
+        <v>0.2721693972014272</v>
       </c>
       <c r="F11" s="3" t="b">
         <v>0</v>
@@ -4192,10 +5012,10 @@
         </is>
       </c>
       <c r="D12" s="3" t="n">
-        <v>-0.3713906763541034</v>
+        <v>-0.2457695761557121</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>0.7199897873752998</v>
+        <v>0.8113736552412463</v>
       </c>
       <c r="F12" s="3" t="b">
         <v>0</v>
@@ -4218,10 +5038,10 @@
         </is>
       </c>
       <c r="D13" s="3" t="n">
-        <v>0.240336707250445</v>
+        <v>0.1196178334243359</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>0.8161134404714866</v>
+        <v>0.907413484953296</v>
       </c>
       <c r="F13" s="3" t="b">
         <v>0</v>
@@ -4244,10 +5064,10 @@
         </is>
       </c>
       <c r="D14" s="3" t="n">
-        <v>0</v>
+        <v>-0.7682212795973759</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>1</v>
+        <v>0.462036004631047</v>
       </c>
       <c r="F14" s="3" t="b">
         <v>0</v>
@@ -4278,10 +5098,10 @@
         </is>
       </c>
       <c r="D16" s="3" t="n">
-        <v>1.344361034193523</v>
+        <v>1.154863252469875</v>
       </c>
       <c r="E16" s="3" t="n">
-        <v>0.2274282079155049</v>
+        <v>0.2860427306908723</v>
       </c>
       <c r="F16" s="3" t="b">
         <v>0</v>
@@ -4300,14 +5120,14 @@
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>Wilcoxon</t>
+          <t>T-test</t>
         </is>
       </c>
       <c r="D17" s="3" t="n">
-        <v>9</v>
+        <v>1.488558185333922</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>0.84375</v>
+        <v>0.1802093661549571</v>
       </c>
       <c r="F17" s="3" t="b">
         <v>0</v>
@@ -4330,10 +5150,10 @@
         </is>
       </c>
       <c r="D18" s="3" t="n">
-        <v>1.222631418787729</v>
+        <v>1.516108590071161</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>0.2673114535246533</v>
+        <v>0.173272933287916</v>
       </c>
       <c r="F18" s="3" t="b">
         <v>0</v>
@@ -4356,10 +5176,10 @@
         </is>
       </c>
       <c r="D19" s="3" t="n">
-        <v>1.757315203104789</v>
+        <v>2.194742847517379</v>
       </c>
       <c r="E19" s="3" t="n">
-        <v>0.1293748508953314</v>
+        <v>0.06422751021232899</v>
       </c>
       <c r="F19" s="3" t="b">
         <v>0</v>
@@ -4390,10 +5210,10 @@
         </is>
       </c>
       <c r="D21" s="3" t="n">
-        <v>1.197148331910294</v>
+        <v>1.511857892036909</v>
       </c>
       <c r="E21" s="3" t="n">
-        <v>0.270212591389518</v>
+        <v>0.1690202030191699</v>
       </c>
       <c r="F21" s="3" t="b">
         <v>0</v>
@@ -4416,10 +5236,10 @@
         </is>
       </c>
       <c r="D22" s="3" t="n">
-        <v>0.4349588362008398</v>
+        <v>0.9386465089278639</v>
       </c>
       <c r="E22" s="3" t="n">
-        <v>0.676686935028977</v>
+        <v>0.3753826881533281</v>
       </c>
       <c r="F22" s="3" t="b">
         <v>0</v>
@@ -4442,10 +5262,10 @@
         </is>
       </c>
       <c r="D23" s="3" t="n">
-        <v>-0.7637626158259733</v>
+        <v>1.615136840834158e-16</v>
       </c>
       <c r="E23" s="3" t="n">
-        <v>0.4699636420584196</v>
+        <v>0.9999999999999999</v>
       </c>
       <c r="F23" s="3" t="b">
         <v>0</v>
@@ -4464,14 +5284,14 @@
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>T-test</t>
+          <t>Wilcoxon</t>
         </is>
       </c>
       <c r="D24" s="3" t="n">
-        <v>1.9296124624699</v>
+        <v>2</v>
       </c>
       <c r="E24" s="3" t="n">
-        <v>0.094976492435775</v>
+        <v>0.0625</v>
       </c>
       <c r="F24" s="3" t="b">
         <v>0</v>
@@ -4502,10 +5322,10 @@
         </is>
       </c>
       <c r="D26" s="3" t="n">
-        <v>1.229232775294831</v>
+        <v>1.711967393494752</v>
       </c>
       <c r="E26" s="3" t="n">
-        <v>0.2586973904995958</v>
+        <v>0.1252618321782634</v>
       </c>
       <c r="F26" s="3" t="b">
         <v>0</v>
@@ -4528,10 +5348,10 @@
         </is>
       </c>
       <c r="D27" s="3" t="n">
-        <v>3.517568943509836</v>
+        <v>3.772968873135195</v>
       </c>
       <c r="E27" s="3" t="n">
-        <v>0.009759500959109107</v>
+        <v>0.005442513014672294</v>
       </c>
       <c r="F27" s="3" t="b">
         <v>1</v>
@@ -4554,10 +5374,10 @@
         </is>
       </c>
       <c r="D28" s="3" t="n">
-        <v>2.861426353911546</v>
+        <v>2.71312556440493</v>
       </c>
       <c r="E28" s="3" t="n">
-        <v>0.02428798676342096</v>
+        <v>0.02652944444936958</v>
       </c>
       <c r="F28" s="3" t="b">
         <v>1</v>
@@ -4580,10 +5400,10 @@
         </is>
       </c>
       <c r="D29" s="3" t="n">
-        <v>4.630064794363034</v>
+        <v>4.850712500726661</v>
       </c>
       <c r="E29" s="3" t="n">
-        <v>0.002397503591143557</v>
+        <v>0.001270703252489122</v>
       </c>
       <c r="F29" s="3" t="b">
         <v>1</v>
@@ -4614,10 +5434,10 @@
         </is>
       </c>
       <c r="D31" s="3" t="n">
-        <v>0.1179682202715451</v>
+        <v>-0.2229112850301412</v>
       </c>
       <c r="E31" s="3" t="n">
-        <v>0.9094065494908765</v>
+        <v>0.8291907476312349</v>
       </c>
       <c r="F31" s="3" t="b">
         <v>0</v>
@@ -4640,10 +5460,10 @@
         </is>
       </c>
       <c r="D32" s="3" t="n">
-        <v>8.5</v>
+        <v>10.5</v>
       </c>
       <c r="E32" s="3" t="n">
-        <v>0.203125</v>
+        <v>0.1796875</v>
       </c>
       <c r="F32" s="3" t="b">
         <v>0</v>
@@ -4666,10 +5486,10 @@
         </is>
       </c>
       <c r="D33" s="3" t="n">
-        <v>-0.7008766440504623</v>
+        <v>-0.9565217391304343</v>
       </c>
       <c r="E33" s="3" t="n">
-        <v>0.5060027660022388</v>
+        <v>0.3668169851556382</v>
       </c>
       <c r="F33" s="3" t="b">
         <v>0</v>
@@ -4688,14 +5508,14 @@
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>T-test</t>
+          <t>Wilcoxon</t>
         </is>
       </c>
       <c r="D34" s="3" t="n">
-        <v>1.297223207936515</v>
+        <v>9</v>
       </c>
       <c r="E34" s="3" t="n">
-        <v>0.2356695290289083</v>
+        <v>0.4375</v>
       </c>
       <c r="F34" s="3" t="b">
         <v>0</v>

</xml_diff>